<commit_message>
Latest sales and corrections for chanderi
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D71F876-72BD-6A4B-B550-68B68D9082B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BEC430-30A1-8749-9F7B-35009014FB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">INVENTORY!$A$1:$T$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Purchases!$A$1:$D$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$212</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2387" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2402" uniqueCount="960">
   <si>
     <t>Notes:</t>
   </si>
@@ -2405,10 +2405,6 @@
     <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200, Black/Golden yellow - Kavya(Kasargod) - 1200, Back/Yellow - Subha - 1200</t>
   </si>
   <si>
-    <t>Bottle Green/Golden Yellow - 2 
-Navy Blue/Bottle Green - 2</t>
-  </si>
-  <si>
     <t>CHR-147</t>
   </si>
   <si>
@@ -2914,12 +2910,6 @@
     <t>Chanderi Silk Saree (Maroon - CHR-119)</t>
   </si>
   <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>Matka Green/Yellow &amp; Bengal Cotton (Adv:1100)</t>
-  </si>
-  <si>
     <t>Simi Sudhir</t>
   </si>
   <si>
@@ -2929,12 +2919,34 @@
     <t>Revathi, Simi Sudhir</t>
   </si>
   <si>
+    <t>Shaino Benny</t>
+  </si>
+  <si>
+    <t>Supriya</t>
+  </si>
+  <si>
+    <t>Chanderi Silk Saree (Green- CHR-119)</t>
+  </si>
+  <si>
+    <t>Mercy Reji</t>
+  </si>
+  <si>
+    <t>Matka Green/Yellow</t>
+  </si>
+  <si>
+    <t>Bottle Green/Golden Yellow - 1
+Navy Blue/Bottle Green - 2</t>
+  </si>
+  <si>
+    <t>Kalaisari (Dharmapuri)</t>
+  </si>
+  <si>
     <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
-Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Unknown - Navy blue, Simi Sudhir - Navy Blue</t>
+Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green</t>
   </si>
   <si>
     <t xml:space="preserve">
-Blue (2), mustard yellow (1), Green (2), Maroon (1), off white (1), Orange (1), Black(5), White(5)</t>
+Blue (2), mustard yellow (1), Maroon (1), off white (1), Orange (1), Black(4), White(5)</t>
   </si>
 </sst>
 </file>
@@ -3847,7 +3859,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>204</c:v>
+                  <c:v>208</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>86</c:v>
@@ -3950,7 +3962,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>68</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>59</c:v>
@@ -4283,7 +4295,7 @@
                   <c:v>61609</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45010.17</c:v>
+                  <c:v>43034.31</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1357</c:v>
@@ -4767,13 +4779,13 @@
                   <c:v>16248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>55936</c:v>
+                  <c:v>55237</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>53524</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7046</c:v>
+                  <c:v>9144</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5207,13 +5219,13 @@
                   <c:v>-5924</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-15066</c:v>
+                  <c:v>-15765</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>49075</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7046</c:v>
+                  <c:v>9144</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5680,10 +5692,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>293</c:v>
+                  <c:v>297</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>131</c:v>
+                  <c:v>127</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6870,7 +6882,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>341464</v>
+        <v>344762</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6887,7 +6899,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>363318</v>
+        <v>364717</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6904,7 +6916,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-13278</v>
+        <v>-9980</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7116,15 +7128,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>283365</v>
+        <v>286663</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>113844.09759999999</v>
+        <v>114943.65079999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>169520.90240000002</v>
+        <v>171719.3492</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7132,11 +7144,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>32210.876400000008</v>
+        <v>34409.323199999984</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹32,211</v>
+        <v>Pay ₹34,409</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7150,11 +7162,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>113775.8048</v>
+        <v>114874.69839999999</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-68206.804799999998</v>
+        <v>-69305.698399999994</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7162,11 +7174,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>3380.2372000000032</v>
+        <v>2281.3436000000074</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹3,380</v>
+        <v>Pay ₹2,281</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7180,11 +7192,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>113844.09759999999</v>
+        <v>114943.65079999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-101314.09759999999</v>
+        <v>-102413.65079999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7192,11 +7204,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-35591.113599999982</v>
+        <v>-36690.666799999977</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹35,591</v>
+        <v>Receive ₹36,691</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7324,7 +7336,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>341464</v>
+        <v>344762</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7333,14 +7345,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-13278</v>
+        <v>-9980</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>98672.37</v>
+        <v>96696.50999999998</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7392,7 +7404,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7416,7 +7428,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7446,11 +7458,11 @@
       </c>
       <c r="C13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>55936</v>
+        <v>55237</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>-15066</v>
+        <v>-15765</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7480,11 +7492,11 @@
       </c>
       <c r="C15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A15)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>7046</v>
+        <v>9144</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>7046</v>
+        <v>9144</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -7612,11 +7624,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -7643,7 +7655,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>45010.17</v>
+        <v>43034.31</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -14678,7 +14690,7 @@
       <c r="F149" s="49"/>
       <c r="G149" s="49"/>
       <c r="H149" s="51" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="I149" s="49" t="s">
         <v>142</v>
@@ -14951,7 +14963,7 @@
       <c r="F160" s="56"/>
       <c r="G160" s="56"/>
       <c r="H160" s="57" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="I160" s="53" t="s">
         <v>341</v>
@@ -15143,7 +15155,7 @@
       <c r="F168" s="49"/>
       <c r="G168" s="49"/>
       <c r="H168" s="51" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="I168" s="49" t="s">
         <v>341</v>
@@ -15428,7 +15440,7 @@
         <v>380</v>
       </c>
       <c r="C180" s="50">
-        <v>1899</v>
+        <v>1200</v>
       </c>
       <c r="D180" s="49" t="s">
         <v>156</v>
@@ -15439,10 +15451,10 @@
       <c r="F180" s="49"/>
       <c r="G180" s="49"/>
       <c r="H180" s="51" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="I180" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="181" spans="1:9" ht="13.5" customHeight="1">
@@ -15871,7 +15883,7 @@
         <v>46168</v>
       </c>
       <c r="B198" s="53" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="C198" s="54">
         <v>5200</v>
@@ -15885,7 +15897,7 @@
       <c r="F198" s="56"/>
       <c r="G198" s="56"/>
       <c r="H198" s="57" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="I198" s="53" t="s">
         <v>142</v>
@@ -15896,7 +15908,7 @@
         <v>46172</v>
       </c>
       <c r="B199" s="49" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="C199" s="50">
         <v>1425</v>
@@ -15910,7 +15922,7 @@
       <c r="F199" s="49"/>
       <c r="G199" s="49"/>
       <c r="H199" s="51" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="I199" s="49" t="s">
         <v>341</v>
@@ -15921,7 +15933,7 @@
         <v>46173</v>
       </c>
       <c r="B200" s="53" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="C200" s="54">
         <v>2850</v>
@@ -15935,7 +15947,7 @@
       <c r="F200" s="56"/>
       <c r="G200" s="56"/>
       <c r="H200" s="57" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="I200" s="53" t="s">
         <v>341</v>
@@ -15946,7 +15958,7 @@
         <v>46173</v>
       </c>
       <c r="B201" s="49" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="C201" s="50">
         <v>2850</v>
@@ -15960,7 +15972,7 @@
       <c r="F201" s="49"/>
       <c r="G201" s="49"/>
       <c r="H201" s="51" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="I201" s="49" t="s">
         <v>341</v>
@@ -15971,7 +15983,7 @@
         <v>46173</v>
       </c>
       <c r="B202" s="53" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="C202" s="54">
         <v>930</v>
@@ -15985,7 +15997,7 @@
       <c r="F202" s="56"/>
       <c r="G202" s="56"/>
       <c r="H202" s="57" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="I202" s="53" t="s">
         <v>341</v>
@@ -15996,7 +16008,7 @@
         <v>46173</v>
       </c>
       <c r="B203" s="49" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C203" s="50">
         <v>930</v>
@@ -16010,7 +16022,7 @@
       <c r="F203" s="49"/>
       <c r="G203" s="49"/>
       <c r="H203" s="51" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="I203" s="49" t="s">
         <v>341</v>
@@ -16021,7 +16033,7 @@
         <v>46175</v>
       </c>
       <c r="B204" s="53" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="C204" s="54">
         <v>699</v>
@@ -16035,7 +16047,7 @@
       <c r="F204" s="56"/>
       <c r="G204" s="56"/>
       <c r="H204" s="57" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="I204" s="53" t="s">
         <v>142</v>
@@ -16046,7 +16058,7 @@
         <v>46175</v>
       </c>
       <c r="B205" s="49" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C205" s="50">
         <v>700</v>
@@ -16060,7 +16072,7 @@
       <c r="F205" s="49"/>
       <c r="G205" s="49"/>
       <c r="H205" s="51" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="I205" s="49" t="s">
         <v>142</v>
@@ -16071,7 +16083,7 @@
         <v>46175</v>
       </c>
       <c r="B206" s="53" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="C206" s="54">
         <v>1350</v>
@@ -16085,7 +16097,7 @@
       <c r="F206" s="56"/>
       <c r="G206" s="56"/>
       <c r="H206" s="51" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="I206" s="53" t="s">
         <v>142</v>
@@ -16096,7 +16108,7 @@
         <v>46175</v>
       </c>
       <c r="B207" s="49" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="C207" s="50">
         <v>699</v>
@@ -16110,7 +16122,7 @@
       <c r="F207" s="49"/>
       <c r="G207" s="49"/>
       <c r="H207" s="51" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="I207" s="49" t="s">
         <v>142</v>
@@ -16121,7 +16133,7 @@
         <v>46175</v>
       </c>
       <c r="B208" s="53" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="C208" s="54">
         <v>699</v>
@@ -16135,7 +16147,7 @@
       <c r="F208" s="56"/>
       <c r="G208" s="56"/>
       <c r="H208" s="57" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="I208" s="53" t="s">
         <v>142</v>
@@ -16146,7 +16158,7 @@
         <v>46176</v>
       </c>
       <c r="B209" s="49" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="C209" s="50">
         <v>699</v>
@@ -16160,7 +16172,7 @@
       <c r="F209" s="49"/>
       <c r="G209" s="49"/>
       <c r="H209" s="51" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="I209" s="49" t="s">
         <v>142</v>
@@ -16171,7 +16183,7 @@
         <v>46176</v>
       </c>
       <c r="B210" s="53" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="C210" s="54">
         <v>2200</v>
@@ -16185,44 +16197,86 @@
       <c r="F210" s="56"/>
       <c r="G210" s="56"/>
       <c r="H210" s="57" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="211" spans="1:9">
-      <c r="A211" s="48"/>
-      <c r="B211" s="49"/>
-      <c r="C211" s="50"/>
-      <c r="D211" s="49"/>
-      <c r="E211" s="49"/>
+    <row r="211" spans="1:9" ht="14">
+      <c r="A211" s="48">
+        <v>46176</v>
+      </c>
+      <c r="B211" s="49" t="s">
+        <v>952</v>
+      </c>
+      <c r="C211" s="50">
+        <v>699</v>
+      </c>
+      <c r="D211" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E211" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F211" s="49"/>
       <c r="G211" s="49"/>
-      <c r="H211" s="51"/>
-      <c r="I211" s="49"/>
+      <c r="H211" s="51" t="s">
+        <v>953</v>
+      </c>
+      <c r="I211" s="49" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="212" spans="1:9">
-      <c r="A212" s="52"/>
-      <c r="B212" s="53"/>
-      <c r="C212" s="54"/>
-      <c r="D212" s="53"/>
-      <c r="E212" s="53"/>
+      <c r="A212" s="52">
+        <v>46176</v>
+      </c>
+      <c r="B212" s="53" t="s">
+        <v>954</v>
+      </c>
+      <c r="C212" s="54">
+        <v>699</v>
+      </c>
+      <c r="D212" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E212" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F212" s="56"/>
       <c r="G212" s="56"/>
-      <c r="H212" s="57"/>
-      <c r="I212" s="53"/>
-    </row>
-    <row r="213" spans="1:9">
-      <c r="A213" s="48"/>
-      <c r="B213" s="49"/>
-      <c r="C213" s="50"/>
-      <c r="D213" s="49"/>
-      <c r="E213" s="49"/>
+      <c r="H212" s="56" t="s">
+        <v>929</v>
+      </c>
+      <c r="I212" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" ht="14">
+      <c r="A213" s="48">
+        <v>46176</v>
+      </c>
+      <c r="B213" s="49" t="s">
+        <v>957</v>
+      </c>
+      <c r="C213" s="50">
+        <v>700</v>
+      </c>
+      <c r="D213" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E213" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F213" s="49"/>
       <c r="G213" s="49"/>
-      <c r="H213" s="51"/>
-      <c r="I213" s="49"/>
+      <c r="H213" s="51" t="s">
+        <v>953</v>
+      </c>
+      <c r="I213" s="49" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="214" spans="1:9">
       <c r="A214" s="52"/>
@@ -16739,7 +16793,7 @@
       <c r="I260" s="59"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I209" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I212" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1260" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -23530,7 +23584,7 @@
         <v>0</v>
       </c>
       <c r="L62" s="66" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="M62" s="66"/>
       <c r="N62" s="66" t="s">
@@ -26582,10 +26636,10 @@
         <v>699</v>
       </c>
       <c r="F120" s="67">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G120" s="67">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H120" s="66">
         <f t="shared" si="9"/>
@@ -26597,14 +26651,14 @@
       </c>
       <c r="J120" s="66">
         <f t="shared" si="10"/>
-        <v>12987.553333333322</v>
+        <v>14244.413333333321</v>
       </c>
       <c r="K120" s="66">
         <f t="shared" si="11"/>
-        <v>7541.1599999999935</v>
+        <v>6284.2999999999947</v>
       </c>
       <c r="L120" s="66" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="M120" s="66" t="s">
         <v>49</v>
@@ -26614,7 +26668,7 @@
       </c>
       <c r="O120" s="66"/>
       <c r="P120" s="66" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="Q120" s="66"/>
       <c r="R120" s="66"/>
@@ -28670,10 +28724,10 @@
         <v>1200</v>
       </c>
       <c r="F147" s="79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G147" s="79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H147" s="78">
         <f t="shared" si="12"/>
@@ -28685,11 +28739,11 @@
       </c>
       <c r="J147" s="78">
         <f t="shared" si="13"/>
-        <v>4314</v>
+        <v>5033</v>
       </c>
       <c r="K147" s="78">
         <f t="shared" si="14"/>
-        <v>2876</v>
+        <v>2157</v>
       </c>
       <c r="L147" s="69" t="s">
         <v>780</v>
@@ -28700,7 +28754,7 @@
       </c>
       <c r="O147" s="69"/>
       <c r="P147" s="69" t="s">
-        <v>781</v>
+        <v>956</v>
       </c>
       <c r="Q147" s="69"/>
       <c r="R147" s="69"/>
@@ -28709,10 +28763,10 @@
     </row>
     <row r="148" spans="1:20" ht="15" customHeight="1">
       <c r="A148" s="66" t="s">
+        <v>781</v>
+      </c>
+      <c r="B148" s="66" t="s">
         <v>782</v>
-      </c>
-      <c r="B148" s="66" t="s">
-        <v>783</v>
       </c>
       <c r="C148" s="66" t="s">
         <v>95</v>
@@ -28746,7 +28800,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="66" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="M148" s="66"/>
       <c r="N148" s="66" t="s">
@@ -28761,10 +28815,10 @@
     </row>
     <row r="149" spans="1:20" ht="15" customHeight="1">
       <c r="A149" s="69" t="s">
+        <v>784</v>
+      </c>
+      <c r="B149" s="69" t="s">
         <v>785</v>
-      </c>
-      <c r="B149" s="69" t="s">
-        <v>786</v>
       </c>
       <c r="C149" s="69" t="s">
         <v>95</v>
@@ -28798,7 +28852,7 @@
         <v>1024</v>
       </c>
       <c r="L149" s="69" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="M149" s="69"/>
       <c r="N149" s="69" t="s">
@@ -28813,10 +28867,10 @@
     </row>
     <row r="150" spans="1:20" ht="15" customHeight="1">
       <c r="A150" s="66" t="s">
+        <v>787</v>
+      </c>
+      <c r="B150" s="66" t="s">
         <v>788</v>
-      </c>
-      <c r="B150" s="66" t="s">
-        <v>789</v>
       </c>
       <c r="C150" s="66" t="s">
         <v>95</v>
@@ -28863,10 +28917,10 @@
     </row>
     <row r="151" spans="1:20" ht="15" customHeight="1">
       <c r="A151" s="69" t="s">
+        <v>789</v>
+      </c>
+      <c r="B151" s="69" t="s">
         <v>790</v>
-      </c>
-      <c r="B151" s="69" t="s">
-        <v>791</v>
       </c>
       <c r="C151" s="69" t="s">
         <v>96</v>
@@ -28900,7 +28954,7 @@
         <v>645</v>
       </c>
       <c r="L151" s="69" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="M151" s="69"/>
       <c r="N151" s="69" t="s">
@@ -28910,7 +28964,7 @@
         <v>210</v>
       </c>
       <c r="P151" s="69" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="Q151" s="69"/>
       <c r="R151" s="69"/>
@@ -28919,10 +28973,10 @@
     </row>
     <row r="152" spans="1:20" ht="15" customHeight="1">
       <c r="A152" s="66" t="s">
+        <v>793</v>
+      </c>
+      <c r="B152" s="66" t="s">
         <v>794</v>
-      </c>
-      <c r="B152" s="66" t="s">
-        <v>795</v>
       </c>
       <c r="C152" s="66" t="s">
         <v>97</v>
@@ -28956,17 +29010,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="66" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M152" s="66"/>
       <c r="N152" s="66" t="s">
         <v>510</v>
       </c>
       <c r="O152" s="66" t="s">
+        <v>796</v>
+      </c>
+      <c r="P152" s="66" t="s">
         <v>797</v>
-      </c>
-      <c r="P152" s="66" t="s">
-        <v>798</v>
       </c>
       <c r="Q152" s="66"/>
       <c r="R152" s="66"/>
@@ -28975,10 +29029,10 @@
     </row>
     <row r="153" spans="1:20" ht="15" customHeight="1">
       <c r="A153" s="69" t="s">
+        <v>798</v>
+      </c>
+      <c r="B153" s="69" t="s">
         <v>799</v>
-      </c>
-      <c r="B153" s="69" t="s">
-        <v>800</v>
       </c>
       <c r="C153" s="69" t="s">
         <v>95</v>
@@ -29012,7 +29066,7 @@
         <v>891.5</v>
       </c>
       <c r="L153" s="69" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="M153" s="69"/>
       <c r="N153" s="69" t="s">
@@ -29020,7 +29074,7 @@
       </c>
       <c r="O153" s="69"/>
       <c r="P153" s="69" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="Q153" s="69"/>
       <c r="R153" s="69"/>
@@ -29029,10 +29083,10 @@
     </row>
     <row r="154" spans="1:20" ht="15" customHeight="1">
       <c r="A154" s="66" t="s">
+        <v>802</v>
+      </c>
+      <c r="B154" s="66" t="s">
         <v>803</v>
-      </c>
-      <c r="B154" s="66" t="s">
-        <v>804</v>
       </c>
       <c r="C154" s="66" t="s">
         <v>96</v>
@@ -29066,14 +29120,14 @@
         <v>1898</v>
       </c>
       <c r="L154" s="66" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="M154" s="66"/>
       <c r="N154" s="66" t="s">
         <v>510</v>
       </c>
       <c r="O154" s="66" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="P154" s="66"/>
       <c r="Q154" s="66"/>
@@ -29083,10 +29137,10 @@
     </row>
     <row r="155" spans="1:20" ht="15" customHeight="1">
       <c r="A155" s="69" t="s">
+        <v>806</v>
+      </c>
+      <c r="B155" s="69" t="s">
         <v>807</v>
-      </c>
-      <c r="B155" s="69" t="s">
-        <v>808</v>
       </c>
       <c r="C155" s="69" t="s">
         <v>96</v>
@@ -29125,7 +29179,7 @@
         <v>599</v>
       </c>
       <c r="O155" s="69" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="P155" s="69"/>
       <c r="Q155" s="69"/>
@@ -29135,10 +29189,10 @@
     </row>
     <row r="156" spans="1:20" ht="15" customHeight="1">
       <c r="A156" s="66" t="s">
+        <v>809</v>
+      </c>
+      <c r="B156" s="66" t="s">
         <v>810</v>
-      </c>
-      <c r="B156" s="66" t="s">
-        <v>811</v>
       </c>
       <c r="C156" s="66" t="s">
         <v>96</v>
@@ -29172,14 +29226,14 @@
         <v>2850</v>
       </c>
       <c r="L156" s="66" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="M156" s="66"/>
       <c r="N156" s="66" t="s">
         <v>510</v>
       </c>
       <c r="O156" s="66" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="P156" s="66"/>
       <c r="Q156" s="66"/>
@@ -29189,10 +29243,10 @@
     </row>
     <row r="157" spans="1:20" ht="15" customHeight="1">
       <c r="A157" s="69" t="s">
+        <v>812</v>
+      </c>
+      <c r="B157" s="69" t="s">
         <v>813</v>
-      </c>
-      <c r="B157" s="69" t="s">
-        <v>814</v>
       </c>
       <c r="C157" s="69" t="s">
         <v>96</v>
@@ -29226,14 +29280,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="69" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="M157" s="69"/>
       <c r="N157" s="69" t="s">
         <v>510</v>
       </c>
       <c r="O157" s="69" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="P157" s="69"/>
       <c r="Q157" s="69"/>
@@ -29243,10 +29297,10 @@
     </row>
     <row r="158" spans="1:20" ht="15" customHeight="1">
       <c r="A158" s="66" t="s">
+        <v>816</v>
+      </c>
+      <c r="B158" s="66" t="s">
         <v>817</v>
-      </c>
-      <c r="B158" s="66" t="s">
-        <v>818</v>
       </c>
       <c r="C158" s="66" t="s">
         <v>96</v>
@@ -29280,14 +29334,14 @@
         <v>3356</v>
       </c>
       <c r="L158" s="66" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="M158" s="66"/>
       <c r="N158" s="66" t="s">
         <v>599</v>
       </c>
       <c r="O158" s="66" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="P158" s="66"/>
       <c r="Q158" s="66"/>
@@ -29297,10 +29351,10 @@
     </row>
     <row r="159" spans="1:20" ht="15" customHeight="1">
       <c r="A159" s="69" t="s">
+        <v>820</v>
+      </c>
+      <c r="B159" s="69" t="s">
         <v>821</v>
-      </c>
-      <c r="B159" s="69" t="s">
-        <v>822</v>
       </c>
       <c r="C159" s="69" t="s">
         <v>96</v>
@@ -29334,14 +29388,14 @@
         <v>2517</v>
       </c>
       <c r="L159" s="69" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="M159" s="69"/>
       <c r="N159" s="69" t="s">
         <v>510</v>
       </c>
       <c r="O159" s="69" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="P159" s="69"/>
       <c r="Q159" s="69"/>
@@ -29351,10 +29405,10 @@
     </row>
     <row r="160" spans="1:20" ht="15" customHeight="1">
       <c r="A160" s="66" t="s">
+        <v>824</v>
+      </c>
+      <c r="B160" s="66" t="s">
         <v>825</v>
-      </c>
-      <c r="B160" s="66" t="s">
-        <v>826</v>
       </c>
       <c r="C160" s="66" t="s">
         <v>95</v>
@@ -29403,10 +29457,10 @@
     </row>
     <row r="161" spans="1:20" ht="15" customHeight="1">
       <c r="A161" s="69" t="s">
+        <v>826</v>
+      </c>
+      <c r="B161" s="69" t="s">
         <v>827</v>
-      </c>
-      <c r="B161" s="69" t="s">
-        <v>828</v>
       </c>
       <c r="C161" s="69" t="s">
         <v>95</v>
@@ -29455,10 +29509,10 @@
     </row>
     <row r="162" spans="1:20" ht="15" customHeight="1">
       <c r="A162" s="66" t="s">
+        <v>828</v>
+      </c>
+      <c r="B162" s="66" t="s">
         <v>829</v>
-      </c>
-      <c r="B162" s="66" t="s">
-        <v>830</v>
       </c>
       <c r="C162" s="66" t="s">
         <v>95</v>
@@ -29507,10 +29561,10 @@
     </row>
     <row r="163" spans="1:20" ht="15" customHeight="1">
       <c r="A163" s="69" t="s">
+        <v>830</v>
+      </c>
+      <c r="B163" s="69" t="s">
         <v>831</v>
-      </c>
-      <c r="B163" s="69" t="s">
-        <v>832</v>
       </c>
       <c r="C163" s="69" t="s">
         <v>95</v>
@@ -29557,10 +29611,10 @@
     </row>
     <row r="164" spans="1:20" ht="60" customHeight="1">
       <c r="A164" s="66" t="s">
+        <v>832</v>
+      </c>
+      <c r="B164" s="66" t="s">
         <v>833</v>
-      </c>
-      <c r="B164" s="66" t="s">
-        <v>834</v>
       </c>
       <c r="C164" s="66" t="s">
         <v>95</v>
@@ -29594,7 +29648,7 @@
         <v>1013</v>
       </c>
       <c r="L164" s="66" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="M164" s="66"/>
       <c r="N164" s="66" t="s">
@@ -29602,7 +29656,7 @@
       </c>
       <c r="O164" s="66"/>
       <c r="P164" s="66" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="Q164" s="66"/>
       <c r="R164" s="66"/>
@@ -29611,10 +29665,10 @@
     </row>
     <row r="165" spans="1:20" ht="15" customHeight="1">
       <c r="A165" s="69" t="s">
+        <v>834</v>
+      </c>
+      <c r="B165" s="69" t="s">
         <v>835</v>
-      </c>
-      <c r="B165" s="69" t="s">
-        <v>836</v>
       </c>
       <c r="C165" s="69" t="s">
         <v>95</v>
@@ -29656,7 +29710,7 @@
       </c>
       <c r="O165" s="69"/>
       <c r="P165" s="69" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="Q165" s="69"/>
       <c r="R165" s="69"/>
@@ -29665,10 +29719,10 @@
     </row>
     <row r="166" spans="1:20" ht="15" customHeight="1">
       <c r="A166" s="66" t="s">
+        <v>837</v>
+      </c>
+      <c r="B166" s="66" t="s">
         <v>838</v>
-      </c>
-      <c r="B166" s="66" t="s">
-        <v>839</v>
       </c>
       <c r="C166" s="66" t="s">
         <v>95</v>
@@ -29708,7 +29762,7 @@
       </c>
       <c r="O166" s="66"/>
       <c r="P166" s="66" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="Q166" s="66"/>
       <c r="R166" s="66"/>
@@ -29717,10 +29771,10 @@
     </row>
     <row r="167" spans="1:20" ht="15" customHeight="1">
       <c r="A167" s="69" t="s">
+        <v>840</v>
+      </c>
+      <c r="B167" s="69" t="s">
         <v>841</v>
-      </c>
-      <c r="B167" s="69" t="s">
-        <v>842</v>
       </c>
       <c r="C167" s="69" t="s">
         <v>95</v>
@@ -29754,7 +29808,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="69" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="M167" s="69"/>
       <c r="N167" s="69" t="s">
@@ -29762,7 +29816,7 @@
       </c>
       <c r="O167" s="69"/>
       <c r="P167" s="69" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="Q167" s="69"/>
       <c r="R167" s="69"/>
@@ -29771,10 +29825,10 @@
     </row>
     <row r="168" spans="1:20" ht="15" customHeight="1">
       <c r="A168" s="66" t="s">
+        <v>844</v>
+      </c>
+      <c r="B168" s="66" t="s">
         <v>845</v>
-      </c>
-      <c r="B168" s="66" t="s">
-        <v>846</v>
       </c>
       <c r="C168" s="66" t="s">
         <v>95</v>
@@ -29808,7 +29862,7 @@
         <v>1216</v>
       </c>
       <c r="L168" s="66" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="M168" s="66"/>
       <c r="N168" s="66" t="s">
@@ -29816,7 +29870,7 @@
       </c>
       <c r="O168" s="66"/>
       <c r="P168" s="66" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="Q168" s="66"/>
       <c r="R168" s="66"/>
@@ -29825,10 +29879,10 @@
     </row>
     <row r="169" spans="1:20" ht="15" customHeight="1">
       <c r="A169" s="69" t="s">
+        <v>848</v>
+      </c>
+      <c r="B169" s="69" t="s">
         <v>849</v>
-      </c>
-      <c r="B169" s="69" t="s">
-        <v>850</v>
       </c>
       <c r="C169" s="69" t="s">
         <v>95</v>
@@ -29868,7 +29922,7 @@
       </c>
       <c r="O169" s="69"/>
       <c r="P169" s="69" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="Q169" s="69"/>
       <c r="R169" s="69"/>
@@ -29877,10 +29931,10 @@
     </row>
     <row r="170" spans="1:20" ht="30" customHeight="1">
       <c r="A170" s="66" t="s">
+        <v>851</v>
+      </c>
+      <c r="B170" s="66" t="s">
         <v>852</v>
-      </c>
-      <c r="B170" s="66" t="s">
-        <v>853</v>
       </c>
       <c r="C170" s="66" t="s">
         <v>95</v>
@@ -29914,7 +29968,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="66" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="M170" s="66"/>
       <c r="N170" s="66" t="s">
@@ -29922,7 +29976,7 @@
       </c>
       <c r="O170" s="66"/>
       <c r="P170" s="66" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="Q170" s="66"/>
       <c r="R170" s="66"/>
@@ -29931,10 +29985,10 @@
     </row>
     <row r="171" spans="1:20" ht="31.5" customHeight="1">
       <c r="A171" s="69" t="s">
+        <v>855</v>
+      </c>
+      <c r="B171" s="66" t="s">
         <v>856</v>
-      </c>
-      <c r="B171" s="66" t="s">
-        <v>857</v>
       </c>
       <c r="C171" s="69" t="s">
         <v>95</v>
@@ -29968,7 +30022,7 @@
         <v>0</v>
       </c>
       <c r="L171" s="69" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="M171" s="69"/>
       <c r="N171" s="69" t="s">
@@ -29983,10 +30037,10 @@
     </row>
     <row r="172" spans="1:20" ht="15" customHeight="1">
       <c r="A172" s="66" t="s">
+        <v>858</v>
+      </c>
+      <c r="B172" s="66" t="s">
         <v>859</v>
-      </c>
-      <c r="B172" s="66" t="s">
-        <v>860</v>
       </c>
       <c r="C172" s="66" t="s">
         <v>95</v>
@@ -30020,7 +30074,7 @@
         <v>2094</v>
       </c>
       <c r="L172" s="66" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="M172" s="66"/>
       <c r="N172" s="66" t="s">
@@ -30035,10 +30089,10 @@
     </row>
     <row r="173" spans="1:20" ht="15" customHeight="1">
       <c r="A173" s="69" t="s">
+        <v>860</v>
+      </c>
+      <c r="B173" s="69" t="s">
         <v>861</v>
-      </c>
-      <c r="B173" s="69" t="s">
-        <v>862</v>
       </c>
       <c r="C173" s="69" t="s">
         <v>95</v>
@@ -30087,10 +30141,10 @@
     </row>
     <row r="174" spans="1:20" ht="15" customHeight="1">
       <c r="A174" s="66" t="s">
+        <v>862</v>
+      </c>
+      <c r="B174" s="66" t="s">
         <v>863</v>
-      </c>
-      <c r="B174" s="66" t="s">
-        <v>864</v>
       </c>
       <c r="C174" s="66" t="s">
         <v>95</v>
@@ -30124,7 +30178,7 @@
         <v>0</v>
       </c>
       <c r="L174" s="66" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="M174" s="66"/>
       <c r="N174" s="66" t="s">
@@ -30139,10 +30193,10 @@
     </row>
     <row r="175" spans="1:20" ht="90" customHeight="1">
       <c r="A175" s="69" t="s">
+        <v>865</v>
+      </c>
+      <c r="B175" s="69" t="s">
         <v>866</v>
-      </c>
-      <c r="B175" s="69" t="s">
-        <v>867</v>
       </c>
       <c r="C175" s="69" t="s">
         <v>95</v>
@@ -30176,7 +30230,7 @@
         <v>4887.75</v>
       </c>
       <c r="L175" s="69" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="M175" s="69"/>
       <c r="N175" s="69" t="s">
@@ -30184,7 +30238,7 @@
       </c>
       <c r="O175" s="69"/>
       <c r="P175" s="69" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="Q175" s="69"/>
       <c r="R175" s="69"/>
@@ -30193,10 +30247,10 @@
     </row>
     <row r="176" spans="1:20" ht="24" customHeight="1">
       <c r="A176" s="66" t="s">
+        <v>867</v>
+      </c>
+      <c r="B176" s="66" t="s">
         <v>868</v>
-      </c>
-      <c r="B176" s="66" t="s">
-        <v>869</v>
       </c>
       <c r="C176" s="66" t="s">
         <v>95</v>
@@ -30230,7 +30284,7 @@
         <v>0</v>
       </c>
       <c r="L176" s="66" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="M176" s="66"/>
       <c r="N176" s="66" t="s">
@@ -30245,10 +30299,10 @@
     </row>
     <row r="177" spans="1:20" ht="34" customHeight="1">
       <c r="A177" s="69" t="s">
+        <v>869</v>
+      </c>
+      <c r="B177" s="69" t="s">
         <v>870</v>
-      </c>
-      <c r="B177" s="69" t="s">
-        <v>871</v>
       </c>
       <c r="C177" s="69" t="s">
         <v>95</v>
@@ -30282,7 +30336,7 @@
         <v>0</v>
       </c>
       <c r="L177" s="69" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="M177" s="69"/>
       <c r="N177" s="69" t="s">
@@ -30290,7 +30344,7 @@
       </c>
       <c r="O177" s="69"/>
       <c r="P177" s="69" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="Q177" s="69"/>
       <c r="R177" s="69"/>
@@ -30299,10 +30353,10 @@
     </row>
     <row r="178" spans="1:20" ht="15" customHeight="1">
       <c r="A178" s="66" t="s">
+        <v>872</v>
+      </c>
+      <c r="B178" s="66" t="s">
         <v>873</v>
-      </c>
-      <c r="B178" s="66" t="s">
-        <v>874</v>
       </c>
       <c r="C178" s="66" t="s">
         <v>95</v>
@@ -30336,7 +30390,7 @@
         <v>0</v>
       </c>
       <c r="L178" s="66" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="M178" s="66"/>
       <c r="N178" s="66" t="s">
@@ -30344,7 +30398,7 @@
       </c>
       <c r="O178" s="66"/>
       <c r="P178" s="66" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="Q178" s="66"/>
       <c r="R178" s="66"/>
@@ -30353,10 +30407,10 @@
     </row>
     <row r="179" spans="1:20" ht="30" customHeight="1">
       <c r="A179" s="69" t="s">
+        <v>875</v>
+      </c>
+      <c r="B179" s="69" t="s">
         <v>876</v>
-      </c>
-      <c r="B179" s="69" t="s">
-        <v>877</v>
       </c>
       <c r="C179" s="69" t="s">
         <v>95</v>
@@ -30390,7 +30444,7 @@
         <v>0</v>
       </c>
       <c r="L179" s="69" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="M179" s="69"/>
       <c r="N179" s="69" t="s">
@@ -30398,7 +30452,7 @@
       </c>
       <c r="O179" s="69"/>
       <c r="P179" s="69" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="Q179" s="69"/>
       <c r="R179" s="69"/>
@@ -30407,10 +30461,10 @@
     </row>
     <row r="180" spans="1:20" ht="34" customHeight="1">
       <c r="A180" s="66" t="s">
+        <v>879</v>
+      </c>
+      <c r="B180" s="66" t="s">
         <v>880</v>
-      </c>
-      <c r="B180" s="66" t="s">
-        <v>881</v>
       </c>
       <c r="C180" s="66" t="s">
         <v>95</v>
@@ -30444,7 +30498,7 @@
         <v>0</v>
       </c>
       <c r="L180" s="66" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="M180" s="66"/>
       <c r="N180" s="66" t="s">
@@ -30459,7 +30513,7 @@
     </row>
     <row r="181" spans="1:20" ht="15" customHeight="1">
       <c r="A181" s="69" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B181" s="69"/>
       <c r="C181" s="69"/>
@@ -30483,7 +30537,7 @@
     </row>
     <row r="182" spans="1:20" ht="15" customHeight="1">
       <c r="A182" s="66" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B182" s="66"/>
       <c r="C182" s="66"/>
@@ -30507,7 +30561,7 @@
     </row>
     <row r="183" spans="1:20" ht="15" customHeight="1">
       <c r="A183" s="69" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B183" s="69"/>
       <c r="C183" s="69"/>
@@ -30531,7 +30585,7 @@
     </row>
     <row r="184" spans="1:20" ht="15" customHeight="1">
       <c r="A184" s="66" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B184" s="66"/>
       <c r="C184" s="66"/>
@@ -30555,7 +30609,7 @@
     </row>
     <row r="185" spans="1:20" ht="15" customHeight="1">
       <c r="A185" s="69" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B185" s="69"/>
       <c r="C185" s="69"/>
@@ -30579,7 +30633,7 @@
     </row>
     <row r="186" spans="1:20" ht="15" customHeight="1">
       <c r="A186" s="66" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B186" s="66"/>
       <c r="C186" s="66"/>
@@ -30603,7 +30657,7 @@
     </row>
     <row r="187" spans="1:20" ht="15" customHeight="1">
       <c r="A187" s="69" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B187" s="69"/>
       <c r="C187" s="69"/>
@@ -30627,7 +30681,7 @@
     </row>
     <row r="188" spans="1:20" ht="15" customHeight="1">
       <c r="A188" s="66" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B188" s="66"/>
       <c r="C188" s="66"/>
@@ -34702,7 +34756,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="95" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B1" s="95"/>
     </row>
@@ -34711,7 +34765,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -34743,25 +34797,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="86" t="s">
+        <v>891</v>
+      </c>
+      <c r="C7" s="86" t="s">
         <v>892</v>
       </c>
-      <c r="C7" s="86" t="s">
+      <c r="D7" s="86" t="s">
         <v>893</v>
       </c>
-      <c r="D7" s="86" t="s">
+      <c r="E7" s="86" t="s">
         <v>894</v>
       </c>
-      <c r="E7" s="86" t="s">
+      <c r="F7" s="86" t="s">
         <v>895</v>
       </c>
-      <c r="F7" s="86" t="s">
+      <c r="G7" s="86" t="s">
         <v>896</v>
       </c>
-      <c r="G7" s="86" t="s">
+      <c r="H7" s="86" t="s">
         <v>897</v>
-      </c>
-      <c r="H7" s="86" t="s">
-        <v>898</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -34865,7 +34919,7 @@
     </row>
     <row r="12" spans="1:8" s="90" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="96" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B12" s="96"/>
       <c r="C12" s="96"/>
@@ -34878,13 +34932,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="86" t="s">
+        <v>899</v>
+      </c>
+      <c r="C13" s="86" t="s">
         <v>900</v>
       </c>
-      <c r="C13" s="86" t="s">
+      <c r="D13" s="86" t="s">
         <v>901</v>
-      </c>
-      <c r="D13" s="86" t="s">
-        <v>902</v>
       </c>
       <c r="E13" s="86" t="s">
         <v>99</v>
@@ -34898,7 +34952,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -34916,7 +34970,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -34970,7 +35024,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -34988,7 +35042,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -35006,7 +35060,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -35024,7 +35078,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -35042,7 +35096,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -35078,7 +35132,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -35114,7 +35168,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -35132,7 +35186,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -35215,7 +35269,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
   </sheetData>
@@ -35245,7 +35299,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="93" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="87" customFormat="1" ht="13.5" customHeight="1">
@@ -35253,22 +35307,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="86" t="s">
+        <v>905</v>
+      </c>
+      <c r="C3" s="86" t="s">
+        <v>890</v>
+      </c>
+      <c r="D3" s="86" t="s">
         <v>906</v>
       </c>
-      <c r="C3" s="86" t="s">
-        <v>891</v>
-      </c>
-      <c r="D3" s="86" t="s">
+      <c r="E3" s="86" t="s">
         <v>907</v>
       </c>
-      <c r="E3" s="86" t="s">
+      <c r="F3" s="86" t="s">
         <v>908</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="G3" s="86" t="s">
         <v>909</v>
-      </c>
-      <c r="G3" s="86" t="s">
-        <v>910</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -35277,7 +35331,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>283365</v>
+        <v>286663</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -35285,11 +35339,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>113844.09759999999</v>
+        <v>114943.65079999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>169520.90240000002</v>
+        <v>171719.3492</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35297,7 +35351,7 @@
       </c>
       <c r="G4" s="88">
         <f>E4+F4</f>
-        <v>32210.876400000008</v>
+        <v>34409.323199999984</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -35314,11 +35368,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>113775.8048</v>
+        <v>114874.69839999999</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-68206.804799999998</v>
+        <v>-69305.698399999994</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35326,7 +35380,7 @@
       </c>
       <c r="G5" s="89">
         <f>E5+F5</f>
-        <v>3380.2372000000032</v>
+        <v>2281.3436000000074</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -35343,11 +35397,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>113844.09759999999</v>
+        <v>114943.65079999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-101314.09759999999</v>
+        <v>-102413.65079999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35355,7 +35409,7 @@
       </c>
       <c r="G6" s="88">
         <f>E6+F6</f>
-        <v>-35591.113599999982</v>
+        <v>-36690.666799999977</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -35365,27 +35419,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stocks correction for blue ajrakh, maheswari & ganga-jamuna hidden
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA0668F-0587-AE42-A516-1D92C0DF7564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C4AA3B-FDC8-314D-8B5B-49CF0365A1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2416" uniqueCount="964">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2423" uniqueCount="965">
   <si>
     <t>Notes:</t>
   </si>
@@ -2807,13 +2807,7 @@
     <t>5. Cash Position After Settlements = Over/(Under) + Net Cash Settlements.</t>
   </si>
   <si>
-    <t>Banarasi Green Old design (1000 advance)</t>
-  </si>
-  <si>
     <t>Sungudi (Alice Christy inspired)</t>
-  </si>
-  <si>
-    <t>Salwar maroon single piece M (CHR-78) - 500 advance, 300 pending</t>
   </si>
   <si>
     <t>Revathi</t>
@@ -2959,6 +2953,15 @@
   </si>
   <si>
     <t>Courier covers and butter papers</t>
+  </si>
+  <si>
+    <t>Salwar maroon single piece M (CHR-78)</t>
+  </si>
+  <si>
+    <t>Banarasi Green Old design</t>
+  </si>
+  <si>
+    <t>Postal parcel charges</t>
   </si>
 </sst>
 </file>
@@ -3977,7 +3980,7 @@
                   <c:v>63</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>59</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>4</c:v>
@@ -4304,7 +4307,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>61609</c:v>
+                  <c:v>60714</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>42615.356666666667</c:v>
@@ -4637,7 +4640,7 @@
                   <c:v>4449</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4440</c:v>
+                  <c:v>4524</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -4791,7 +4794,7 @@
                   <c:v>16248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>55267</c:v>
+                  <c:v>54177</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>53524</c:v>
@@ -5231,13 +5234,13 @@
                   <c:v>-5924</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-15735</c:v>
+                  <c:v>-16825</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>49075</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5403</c:v>
+                  <c:v>5319</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5707,7 +5710,7 @@
                   <c:v>298</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>126</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6879,7 +6882,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>359182</v>
+        <v>359266</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -6894,7 +6897,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>346141</v>
+        <v>351391</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6911,7 +6914,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>365446</v>
+        <v>364356</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6928,7 +6931,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-13041</v>
+        <v>-7875</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6963,7 +6966,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>20214.326666666671</v>
+        <v>20270.326666666671</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -6973,7 +6976,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>6970.3366666666698</v>
+        <v>6942.3366666666698</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -6983,7 +6986,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-27184.66333333333</v>
+        <v>-27212.66333333333</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7022,15 +7025,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>158245</v>
+        <v>158329</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>38517.666666666672</v>
+        <v>38573.666666666672</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7038,11 +7041,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>20214.326666666671</v>
+        <v>20270.326666666671</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹20,214</v>
+        <v>Receive ₹20,270</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7056,11 +7059,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>48609.666666666672</v>
+        <v>48581.666666666672</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7068,11 +7071,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>6970.3366666666698</v>
+        <v>6942.3366666666698</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹6,970</v>
+        <v>Receive ₹6,942</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7086,11 +7089,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-87127.333333333328</v>
+        <v>-87155.333333333328</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7098,11 +7101,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-27184.66333333333</v>
+        <v>-27212.66333333333</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹27,185</v>
+        <v>Pay ₹27,213</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7140,15 +7143,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>288042</v>
+        <v>293292</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>115403.40939999999</v>
+        <v>117153.7594</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>172638.5906</v>
+        <v>176138.24060000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7156,11 +7159,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>35328.564599999983</v>
+        <v>38828.214600000007</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹35,329</v>
+        <v>Pay ₹38,828</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7174,11 +7177,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>115334.18119999999</v>
+        <v>117083.48119999999</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-69765.181199999992</v>
+        <v>-71514.481199999995</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7186,11 +7189,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>1821.8608000000095</v>
+        <v>72.560800000006566</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹1,822</v>
+        <v>Pay ₹73</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7204,11 +7207,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>115403.40939999999</v>
+        <v>117153.7594</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-102873.40939999999</v>
+        <v>-104623.7594</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7216,11 +7219,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-37150.425399999978</v>
+        <v>-38900.775399999984</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹37,150</v>
+        <v>Receive ₹38,901</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7332,7 +7335,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46177</v>
+        <v>46178</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7341,14 +7344,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>359182</v>
+        <v>359266</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>346141</v>
+        <v>351391</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7357,7 +7360,7 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-13041</v>
+        <v>-7875</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
@@ -7440,7 +7443,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7470,11 +7473,11 @@
       </c>
       <c r="C13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>55267</v>
+        <v>54177</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>-15735</v>
+        <v>-16825</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7500,7 +7503,7 @@
       </c>
       <c r="B15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A15)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>4440</v>
+        <v>4524</v>
       </c>
       <c r="C15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A15)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
@@ -7508,7 +7511,7 @@
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>5403</v>
+        <v>5319</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -7647,7 +7650,7 @@
       </c>
       <c r="K47" s="31">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$477=J47)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>61609</v>
+        <v>60714</v>
       </c>
     </row>
     <row r="48" spans="6:11" ht="15" customHeight="1">
@@ -7660,7 +7663,7 @@
       </c>
       <c r="H48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J48" s="30" t="s">
         <v>95</v>
@@ -8802,7 +8805,7 @@
         <v>960</v>
       </c>
       <c r="D74" s="36" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15" customHeight="1">
@@ -8830,7 +8833,7 @@
         <v>2900</v>
       </c>
       <c r="D76" s="36" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" customHeight="1">
@@ -8844,14 +8847,22 @@
         <v>180</v>
       </c>
       <c r="D77" s="39" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" customHeight="1">
-      <c r="A78" s="35"/>
-      <c r="B78" s="36"/>
-      <c r="C78" s="37"/>
-      <c r="D78" s="36"/>
+      <c r="A78" s="35">
+        <v>46178</v>
+      </c>
+      <c r="B78" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C78" s="37">
+        <v>84</v>
+      </c>
+      <c r="D78" s="36" t="s">
+        <v>964</v>
+      </c>
     </row>
     <row r="79" spans="1:4" ht="15" customHeight="1">
       <c r="A79" s="38"/>
@@ -14734,7 +14745,7 @@
       <c r="F149" s="49"/>
       <c r="G149" s="49"/>
       <c r="H149" s="51" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="I149" s="49" t="s">
         <v>142</v>
@@ -14996,7 +15007,7 @@
         <v>352</v>
       </c>
       <c r="C160" s="54">
-        <v>1380</v>
+        <v>1000</v>
       </c>
       <c r="D160" s="53" t="s">
         <v>156</v>
@@ -15007,10 +15018,10 @@
       <c r="F160" s="56"/>
       <c r="G160" s="56"/>
       <c r="H160" s="57" t="s">
-        <v>915</v>
+        <v>963</v>
       </c>
       <c r="I160" s="53" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="161" spans="1:9" ht="13.5" customHeight="1">
@@ -15096,9 +15107,11 @@
         <v>209</v>
       </c>
       <c r="C164" s="54">
-        <v>1380</v>
-      </c>
-      <c r="D164" s="53"/>
+        <v>1000</v>
+      </c>
+      <c r="D164" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="E164" s="53" t="s">
         <v>49</v>
       </c>
@@ -15108,7 +15121,7 @@
         <v>358</v>
       </c>
       <c r="I164" s="53" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="165" spans="1:9" ht="13.5" customHeight="1">
@@ -15119,9 +15132,11 @@
         <v>158</v>
       </c>
       <c r="C165" s="50">
-        <v>1380</v>
-      </c>
-      <c r="D165" s="49"/>
+        <v>1200</v>
+      </c>
+      <c r="D165" s="49" t="s">
+        <v>156</v>
+      </c>
       <c r="E165" s="49" t="s">
         <v>49</v>
       </c>
@@ -15131,7 +15146,7 @@
         <v>359</v>
       </c>
       <c r="I165" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="166" spans="1:9" ht="13.5" customHeight="1">
@@ -15167,9 +15182,11 @@
         <v>185</v>
       </c>
       <c r="C167" s="50">
-        <v>1250</v>
-      </c>
-      <c r="D167" s="49"/>
+        <v>1100</v>
+      </c>
+      <c r="D167" s="49" t="s">
+        <v>156</v>
+      </c>
       <c r="E167" s="49" t="s">
         <v>49</v>
       </c>
@@ -15179,7 +15196,7 @@
         <v>362</v>
       </c>
       <c r="I167" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="168" spans="1:9" ht="13.5" customHeight="1">
@@ -15192,17 +15209,19 @@
       <c r="C168" s="50">
         <v>950</v>
       </c>
-      <c r="D168" s="49"/>
+      <c r="D168" s="49" t="s">
+        <v>156</v>
+      </c>
       <c r="E168" s="49" t="s">
         <v>49</v>
       </c>
       <c r="F168" s="49"/>
       <c r="G168" s="49"/>
       <c r="H168" s="51" t="s">
-        <v>917</v>
+        <v>962</v>
       </c>
       <c r="I168" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="169" spans="1:9" ht="13.5" customHeight="1">
@@ -15215,7 +15234,9 @@
       <c r="C169" s="54">
         <v>650</v>
       </c>
-      <c r="D169" s="53"/>
+      <c r="D169" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="E169" s="53" t="s">
         <v>49</v>
       </c>
@@ -15497,7 +15518,7 @@
       <c r="F180" s="49"/>
       <c r="G180" s="49"/>
       <c r="H180" s="51" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="I180" s="49" t="s">
         <v>142</v>
@@ -15929,7 +15950,7 @@
         <v>46168</v>
       </c>
       <c r="B198" s="53" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="C198" s="54">
         <v>5200</v>
@@ -15943,7 +15964,7 @@
       <c r="F198" s="56"/>
       <c r="G198" s="56"/>
       <c r="H198" s="57" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="I198" s="53" t="s">
         <v>142</v>
@@ -15954,7 +15975,7 @@
         <v>46172</v>
       </c>
       <c r="B199" s="49" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="C199" s="50">
         <v>1425</v>
@@ -15968,7 +15989,7 @@
       <c r="F199" s="49"/>
       <c r="G199" s="49"/>
       <c r="H199" s="51" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="I199" s="49" t="s">
         <v>341</v>
@@ -15979,7 +16000,7 @@
         <v>46173</v>
       </c>
       <c r="B200" s="53" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="C200" s="54">
         <v>2850</v>
@@ -15993,7 +16014,7 @@
       <c r="F200" s="56"/>
       <c r="G200" s="56"/>
       <c r="H200" s="57" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="I200" s="53" t="s">
         <v>341</v>
@@ -16004,7 +16025,7 @@
         <v>46173</v>
       </c>
       <c r="B201" s="49" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="C201" s="50">
         <v>2850</v>
@@ -16018,7 +16039,7 @@
       <c r="F201" s="49"/>
       <c r="G201" s="49"/>
       <c r="H201" s="51" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="I201" s="49" t="s">
         <v>341</v>
@@ -16029,7 +16050,7 @@
         <v>46173</v>
       </c>
       <c r="B202" s="53" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="C202" s="54">
         <v>930</v>
@@ -16043,7 +16064,7 @@
       <c r="F202" s="56"/>
       <c r="G202" s="56"/>
       <c r="H202" s="57" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="I202" s="53" t="s">
         <v>341</v>
@@ -16054,7 +16075,7 @@
         <v>46173</v>
       </c>
       <c r="B203" s="49" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="C203" s="50">
         <v>930</v>
@@ -16068,7 +16089,7 @@
       <c r="F203" s="49"/>
       <c r="G203" s="49"/>
       <c r="H203" s="51" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="I203" s="49" t="s">
         <v>341</v>
@@ -16079,7 +16100,7 @@
         <v>46175</v>
       </c>
       <c r="B204" s="53" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="C204" s="54">
         <v>699</v>
@@ -16093,7 +16114,7 @@
       <c r="F204" s="56"/>
       <c r="G204" s="56"/>
       <c r="H204" s="57" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="I204" s="53" t="s">
         <v>142</v>
@@ -16104,7 +16125,7 @@
         <v>46175</v>
       </c>
       <c r="B205" s="49" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="C205" s="50">
         <v>700</v>
@@ -16118,7 +16139,7 @@
       <c r="F205" s="49"/>
       <c r="G205" s="49"/>
       <c r="H205" s="51" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="I205" s="49" t="s">
         <v>142</v>
@@ -16129,7 +16150,7 @@
         <v>46175</v>
       </c>
       <c r="B206" s="53" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="C206" s="54">
         <v>1350</v>
@@ -16143,7 +16164,7 @@
       <c r="F206" s="56"/>
       <c r="G206" s="56"/>
       <c r="H206" s="51" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="I206" s="53" t="s">
         <v>142</v>
@@ -16154,7 +16175,7 @@
         <v>46175</v>
       </c>
       <c r="B207" s="49" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="C207" s="50">
         <v>699</v>
@@ -16168,7 +16189,7 @@
       <c r="F207" s="49"/>
       <c r="G207" s="49"/>
       <c r="H207" s="51" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="I207" s="49" t="s">
         <v>142</v>
@@ -16179,7 +16200,7 @@
         <v>46175</v>
       </c>
       <c r="B208" s="53" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="C208" s="54">
         <v>699</v>
@@ -16193,7 +16214,7 @@
       <c r="F208" s="56"/>
       <c r="G208" s="56"/>
       <c r="H208" s="57" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="I208" s="53" t="s">
         <v>142</v>
@@ -16204,7 +16225,7 @@
         <v>46176</v>
       </c>
       <c r="B209" s="49" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="C209" s="50">
         <v>699</v>
@@ -16218,7 +16239,7 @@
       <c r="F209" s="49"/>
       <c r="G209" s="49"/>
       <c r="H209" s="51" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="I209" s="49" t="s">
         <v>142</v>
@@ -16229,7 +16250,7 @@
         <v>46176</v>
       </c>
       <c r="B210" s="53" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="C210" s="54">
         <v>2200</v>
@@ -16243,7 +16264,7 @@
       <c r="F210" s="56"/>
       <c r="G210" s="56"/>
       <c r="H210" s="57" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>142</v>
@@ -16254,7 +16275,7 @@
         <v>46176</v>
       </c>
       <c r="B211" s="49" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="C211" s="50">
         <v>699</v>
@@ -16268,7 +16289,7 @@
       <c r="F211" s="49"/>
       <c r="G211" s="49"/>
       <c r="H211" s="51" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="I211" s="49" t="s">
         <v>142</v>
@@ -16279,7 +16300,7 @@
         <v>46176</v>
       </c>
       <c r="B212" s="53" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="C212" s="54">
         <v>699</v>
@@ -16293,7 +16314,7 @@
       <c r="F212" s="56"/>
       <c r="G212" s="56"/>
       <c r="H212" s="56" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="I212" s="53" t="s">
         <v>142</v>
@@ -16304,7 +16325,7 @@
         <v>46176</v>
       </c>
       <c r="B213" s="49" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="C213" s="50">
         <v>700</v>
@@ -16318,7 +16339,7 @@
       <c r="F213" s="49"/>
       <c r="G213" s="49"/>
       <c r="H213" s="51" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="I213" s="49" t="s">
         <v>142</v>
@@ -16329,7 +16350,7 @@
         <v>46177</v>
       </c>
       <c r="B214" s="53" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="C214" s="54">
         <v>699</v>
@@ -16343,7 +16364,7 @@
       <c r="F214" s="56"/>
       <c r="G214" s="56"/>
       <c r="H214" s="56" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="I214" s="53" t="s">
         <v>142</v>
@@ -23644,7 +23665,7 @@
         <v>0</v>
       </c>
       <c r="L62" s="66" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="M62" s="66"/>
       <c r="N62" s="66" t="s">
@@ -24843,11 +24864,11 @@
         <v>3</v>
       </c>
       <c r="G85" s="70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H85" s="69">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I85" s="69">
         <f>IF(D85&lt;&gt;"",D85,IFERROR(E85/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -24859,7 +24880,7 @@
       </c>
       <c r="K85" s="69">
         <f t="shared" si="8"/>
-        <v>895</v>
+        <v>0</v>
       </c>
       <c r="L85" s="69" t="s">
         <v>621</v>
@@ -26718,7 +26739,7 @@
         <v>5865.3466666666618</v>
       </c>
       <c r="L120" s="66" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="M120" s="66" t="s">
         <v>49</v>
@@ -26728,7 +26749,7 @@
       </c>
       <c r="O120" s="66"/>
       <c r="P120" s="66" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="Q120" s="66"/>
       <c r="R120" s="66"/>
@@ -28814,7 +28835,7 @@
       </c>
       <c r="O147" s="69"/>
       <c r="P147" s="69" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="Q147" s="69"/>
       <c r="R147" s="69"/>
@@ -29708,7 +29729,7 @@
         <v>1013</v>
       </c>
       <c r="L164" s="66" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="M164" s="66"/>
       <c r="N164" s="66" t="s">
@@ -29716,7 +29737,7 @@
       </c>
       <c r="O164" s="66"/>
       <c r="P164" s="66" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="Q164" s="66"/>
       <c r="R164" s="66"/>
@@ -30134,7 +30155,7 @@
         <v>2094</v>
       </c>
       <c r="L172" s="66" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="M172" s="66"/>
       <c r="N172" s="66" t="s">
@@ -30290,7 +30311,7 @@
         <v>4887.75</v>
       </c>
       <c r="L175" s="69" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="M175" s="69"/>
       <c r="N175" s="69" t="s">
@@ -30298,7 +30319,7 @@
       </c>
       <c r="O175" s="69"/>
       <c r="P175" s="69" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="Q175" s="69"/>
       <c r="R175" s="69"/>
@@ -30344,7 +30365,7 @@
         <v>0</v>
       </c>
       <c r="L176" s="66" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="M176" s="66"/>
       <c r="N176" s="66" t="s">
@@ -30396,7 +30417,7 @@
         <v>0</v>
       </c>
       <c r="L177" s="69" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="M177" s="69"/>
       <c r="N177" s="69" t="s">
@@ -30450,7 +30471,7 @@
         <v>0</v>
       </c>
       <c r="L178" s="66" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="M178" s="66"/>
       <c r="N178" s="66" t="s">
@@ -30558,7 +30579,7 @@
         <v>0</v>
       </c>
       <c r="L180" s="66" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="M180" s="66"/>
       <c r="N180" s="66" t="s">
@@ -34884,15 +34905,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>158245</v>
+        <v>158329</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>38517.666666666672</v>
+        <v>38573.666666666672</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34900,7 +34921,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>38517.666666666672</v>
+        <v>38573.666666666672</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -34908,7 +34929,7 @@
       </c>
       <c r="H8" s="88">
         <f>F8-G8</f>
-        <v>20214.326666666671</v>
+        <v>20270.326666666671</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -34921,11 +34942,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>48609.666666666672</v>
+        <v>48581.666666666672</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34933,7 +34954,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>48609.666666666672</v>
+        <v>48581.666666666672</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -34941,7 +34962,7 @@
       </c>
       <c r="H9" s="89">
         <f>F9-G9</f>
-        <v>6970.3366666666698</v>
+        <v>6942.3366666666698</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -34954,11 +34975,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119727.33333333333</v>
+        <v>119755.33333333333</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-87127.333333333328</v>
+        <v>-87155.333333333328</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34966,7 +34987,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-87127.333333333328</v>
+        <v>-87155.333333333328</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -34974,7 +34995,7 @@
       </c>
       <c r="H10" s="88">
         <f>F10-G10</f>
-        <v>-27184.66333333333</v>
+        <v>-27212.66333333333</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="90" customFormat="1" ht="15.75" customHeight="1">
@@ -35391,7 +35412,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>288042</v>
+        <v>293292</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -35399,11 +35420,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>115403.40939999999</v>
+        <v>117153.7594</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>172638.5906</v>
+        <v>176138.24060000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35411,7 +35432,7 @@
       </c>
       <c r="G4" s="88">
         <f>E4+F4</f>
-        <v>35328.564599999983</v>
+        <v>38828.214600000007</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -35428,11 +35449,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>115334.18119999999</v>
+        <v>117083.48119999999</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-69765.181199999992</v>
+        <v>-71514.481199999995</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35440,7 +35461,7 @@
       </c>
       <c r="G5" s="89">
         <f>E5+F5</f>
-        <v>1821.8608000000095</v>
+        <v>72.560800000006566</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -35457,11 +35478,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>115403.40939999999</v>
+        <v>117153.7594</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-102873.40939999999</v>
+        <v>-104623.7594</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35469,7 +35490,7 @@
       </c>
       <c r="G6" s="88">
         <f>E6+F6</f>
-        <v>-37150.425399999978</v>
+        <v>-38900.775399999984</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Sales updates by Susmi
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{128BE14C-F788-4747-9C4B-4951ACAA3A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C1FD16-9354-0C4D-BD3C-A24F32FA3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2423" uniqueCount="965">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="966">
   <si>
     <t>Notes:</t>
   </si>
@@ -2864,9 +2864,6 @@
     <t>Grey-Black/Red</t>
   </si>
   <si>
-    <t>Matka (peacock blue/maroon CHR-174), Narayanpett purple/bottle green (CHR-163)</t>
-  </si>
-  <si>
     <t>Peacok Blue/Maroon - 2
 Purple/Green - 1
 Navy Blue/Maroon - 2
@@ -2962,6 +2959,12 @@
   </si>
   <si>
     <t>Postal parcel charges</t>
+  </si>
+  <si>
+    <t>Matka (peacock blue/maroon CHR-174), Narayanpett purple/bottle green (CHR-163), Ganga Jamuna (CHR-140)</t>
+  </si>
+  <si>
+    <t>Jaimy (1000)</t>
   </si>
 </sst>
 </file>
@@ -3874,7 +3877,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>209</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>86</c:v>
@@ -3977,7 +3980,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>63</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>58</c:v>
@@ -4310,7 +4313,7 @@
                   <c:v>60714</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>42615.356666666667</c:v>
+                  <c:v>41777.356666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1357</c:v>
@@ -4797,7 +4800,7 @@
                   <c:v>54177</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>53524</c:v>
+                  <c:v>54524</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>9843</c:v>
@@ -5237,7 +5240,7 @@
                   <c:v>-16825</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>49075</c:v>
+                  <c:v>50075</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>5319</c:v>
@@ -5707,10 +5710,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>298</c:v>
+                  <c:v>299</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>125</c:v>
+                  <c:v>124</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6897,7 +6900,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>351391</v>
+        <v>359021</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -6914,7 +6917,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>364356</v>
+        <v>365356</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -6931,7 +6934,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-7875</v>
+        <v>-245</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7147,11 +7150,11 @@
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>117153.7594</v>
+        <v>119697.60139999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>176138.24060000002</v>
+        <v>173594.39860000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7159,11 +7162,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>38828.214600000007</v>
+        <v>36284.372600000002</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹38,828</v>
+        <v>Pay ₹36,284</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7173,15 +7176,15 @@
       </c>
       <c r="B27" s="12">
         <f>'Cash Pool'!B5</f>
-        <v>45569</v>
+        <v>53199</v>
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>117083.48119999999</v>
+        <v>119625.7972</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-71514.481199999995</v>
+        <v>-66426.797200000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7189,11 +7192,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>72.560800000006566</v>
+        <v>5160.2448000000004</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹73</v>
+        <v>Pay ₹5,160</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7207,11 +7210,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>117153.7594</v>
+        <v>119697.60139999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-104623.7594</v>
+        <v>-107167.60139999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7219,11 +7222,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-38900.775399999984</v>
+        <v>-41444.617399999974</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹38,901</v>
+        <v>Receive ₹41,445</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7351,7 +7354,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>351391</v>
+        <v>359021</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7360,14 +7363,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-7875</v>
+        <v>-245</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>96277.556666666656</v>
+        <v>95439.556666666656</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7419,7 +7422,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7443,7 +7446,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7490,11 +7493,11 @@
       </c>
       <c r="C14" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A14)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>53524</v>
+        <v>54524</v>
       </c>
       <c r="D14" s="21">
         <f t="shared" si="0"/>
-        <v>49075</v>
+        <v>50075</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1">
@@ -7639,11 +7642,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -7670,7 +7673,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>42615.356666666667</v>
+        <v>41777.356666666667</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -8805,7 +8808,7 @@
         <v>960</v>
       </c>
       <c r="D74" s="36" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15" customHeight="1">
@@ -8833,7 +8836,7 @@
         <v>2900</v>
       </c>
       <c r="D76" s="36" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="15" customHeight="1">
@@ -8847,7 +8850,7 @@
         <v>180</v>
       </c>
       <c r="D77" s="39" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15" customHeight="1">
@@ -8861,7 +8864,7 @@
         <v>84</v>
       </c>
       <c r="D78" s="36" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" customHeight="1">
@@ -15018,7 +15021,7 @@
       <c r="F160" s="56"/>
       <c r="G160" s="56"/>
       <c r="H160" s="57" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="I160" s="53" t="s">
         <v>142</v>
@@ -15218,7 +15221,7 @@
       <c r="F168" s="49"/>
       <c r="G168" s="49"/>
       <c r="H168" s="51" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="I168" s="49" t="s">
         <v>142</v>
@@ -15518,7 +15521,7 @@
       <c r="F180" s="49"/>
       <c r="G180" s="49"/>
       <c r="H180" s="51" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="I180" s="49" t="s">
         <v>142</v>
@@ -16014,13 +16017,13 @@
       <c r="F200" s="56"/>
       <c r="G200" s="56"/>
       <c r="H200" s="57" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="I200" s="53" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="201" spans="1:9" ht="28">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" ht="42">
       <c r="A201" s="48">
         <v>46173</v>
       </c>
@@ -16028,7 +16031,7 @@
         <v>930</v>
       </c>
       <c r="C201" s="50">
-        <v>2850</v>
+        <v>3850</v>
       </c>
       <c r="D201" s="49" t="s">
         <v>144</v>
@@ -16039,10 +16042,10 @@
       <c r="F201" s="49"/>
       <c r="G201" s="49"/>
       <c r="H201" s="51" t="s">
-        <v>934</v>
+        <v>964</v>
       </c>
       <c r="I201" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="202" spans="1:9" ht="14">
@@ -16067,7 +16070,7 @@
         <v>925</v>
       </c>
       <c r="I202" s="53" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="203" spans="1:9" ht="14">
@@ -16100,7 +16103,7 @@
         <v>46175</v>
       </c>
       <c r="B204" s="53" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="C204" s="54">
         <v>699</v>
@@ -16125,7 +16128,7 @@
         <v>46175</v>
       </c>
       <c r="B205" s="49" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="C205" s="50">
         <v>700</v>
@@ -16139,7 +16142,7 @@
       <c r="F205" s="49"/>
       <c r="G205" s="49"/>
       <c r="H205" s="51" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="I205" s="49" t="s">
         <v>142</v>
@@ -16150,7 +16153,7 @@
         <v>46175</v>
       </c>
       <c r="B206" s="53" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="C206" s="54">
         <v>1350</v>
@@ -16164,7 +16167,7 @@
       <c r="F206" s="56"/>
       <c r="G206" s="56"/>
       <c r="H206" s="51" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="I206" s="53" t="s">
         <v>142</v>
@@ -16175,7 +16178,7 @@
         <v>46175</v>
       </c>
       <c r="B207" s="49" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="C207" s="50">
         <v>699</v>
@@ -16189,7 +16192,7 @@
       <c r="F207" s="49"/>
       <c r="G207" s="49"/>
       <c r="H207" s="51" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="I207" s="49" t="s">
         <v>142</v>
@@ -16200,7 +16203,7 @@
         <v>46175</v>
       </c>
       <c r="B208" s="53" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C208" s="54">
         <v>699</v>
@@ -16214,7 +16217,7 @@
       <c r="F208" s="56"/>
       <c r="G208" s="56"/>
       <c r="H208" s="57" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="I208" s="53" t="s">
         <v>142</v>
@@ -16225,7 +16228,7 @@
         <v>46176</v>
       </c>
       <c r="B209" s="49" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="C209" s="50">
         <v>699</v>
@@ -16239,7 +16242,7 @@
       <c r="F209" s="49"/>
       <c r="G209" s="49"/>
       <c r="H209" s="51" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="I209" s="49" t="s">
         <v>142</v>
@@ -16250,7 +16253,7 @@
         <v>46176</v>
       </c>
       <c r="B210" s="53" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C210" s="54">
         <v>2200</v>
@@ -16264,7 +16267,7 @@
       <c r="F210" s="56"/>
       <c r="G210" s="56"/>
       <c r="H210" s="57" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="I210" s="53" t="s">
         <v>142</v>
@@ -16275,7 +16278,7 @@
         <v>46176</v>
       </c>
       <c r="B211" s="49" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="C211" s="50">
         <v>699</v>
@@ -16289,7 +16292,7 @@
       <c r="F211" s="49"/>
       <c r="G211" s="49"/>
       <c r="H211" s="51" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="I211" s="49" t="s">
         <v>142</v>
@@ -16300,7 +16303,7 @@
         <v>46176</v>
       </c>
       <c r="B212" s="53" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="C212" s="54">
         <v>699</v>
@@ -16325,7 +16328,7 @@
         <v>46176</v>
       </c>
       <c r="B213" s="49" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="C213" s="50">
         <v>700</v>
@@ -16339,7 +16342,7 @@
       <c r="F213" s="49"/>
       <c r="G213" s="49"/>
       <c r="H213" s="51" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="I213" s="49" t="s">
         <v>142</v>
@@ -16350,7 +16353,7 @@
         <v>46177</v>
       </c>
       <c r="B214" s="53" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="C214" s="54">
         <v>699</v>
@@ -26739,7 +26742,7 @@
         <v>5865.3466666666618</v>
       </c>
       <c r="L120" s="66" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="M120" s="66" t="s">
         <v>49</v>
@@ -26749,7 +26752,7 @@
       </c>
       <c r="O120" s="66"/>
       <c r="P120" s="66" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="Q120" s="66"/>
       <c r="R120" s="66"/>
@@ -28495,10 +28498,10 @@
         <v>1100</v>
       </c>
       <c r="F141" s="79">
+        <v>1</v>
+      </c>
+      <c r="G141" s="79">
         <v>0</v>
-      </c>
-      <c r="G141" s="79">
-        <v>1</v>
       </c>
       <c r="H141" s="78">
         <f t="shared" si="12"/>
@@ -28510,16 +28513,18 @@
       </c>
       <c r="J141" s="78">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>838</v>
       </c>
       <c r="K141" s="78">
         <f t="shared" si="14"/>
-        <v>838</v>
-      </c>
-      <c r="L141" s="69"/>
+        <v>0</v>
+      </c>
+      <c r="L141" s="69" t="s">
+        <v>965</v>
+      </c>
       <c r="M141" s="69"/>
       <c r="N141" s="69" t="s">
-        <v>599</v>
+        <v>425</v>
       </c>
       <c r="O141" s="69"/>
       <c r="P141" s="69"/>
@@ -28835,7 +28840,7 @@
       </c>
       <c r="O147" s="69"/>
       <c r="P147" s="69" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="Q147" s="69"/>
       <c r="R147" s="69"/>
@@ -30155,7 +30160,7 @@
         <v>2094</v>
       </c>
       <c r="L172" s="66" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="M172" s="66"/>
       <c r="N172" s="66" t="s">
@@ -30319,7 +30324,7 @@
       </c>
       <c r="O175" s="69"/>
       <c r="P175" s="69" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="Q175" s="69"/>
       <c r="R175" s="69"/>
@@ -35420,11 +35425,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>117153.7594</v>
+        <v>119697.60139999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>176138.24060000002</v>
+        <v>173594.39860000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35432,7 +35437,7 @@
       </c>
       <c r="G4" s="88">
         <f>E4+F4</f>
-        <v>38828.214600000007</v>
+        <v>36284.372600000002</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -35441,7 +35446,7 @@
       </c>
       <c r="B5" s="11">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A5,Sales!$I:$I,"Completed"),0)</f>
-        <v>45569</v>
+        <v>53199</v>
       </c>
       <c r="C5" s="11">
         <f>VLOOKUP($A5,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -35449,11 +35454,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>117083.48119999999</v>
+        <v>119625.7972</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-71514.481199999995</v>
+        <v>-66426.797200000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35461,7 +35466,7 @@
       </c>
       <c r="G5" s="89">
         <f>E5+F5</f>
-        <v>72.560800000006566</v>
+        <v>5160.2448000000004</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -35478,11 +35483,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>117153.7594</v>
+        <v>119697.60139999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-104623.7594</v>
+        <v>-107167.60139999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -35490,7 +35495,7 @@
       </c>
       <c r="G6" s="88">
         <f>E6+F6</f>
-        <v>-38900.775399999984</v>
+        <v>-41444.617399999974</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
June 6 parcel charges
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C1FD16-9354-0C4D-BD3C-A24F32FA3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D858E6E-A89D-4045-BCA2-565636D81419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="966">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2426" uniqueCount="966">
   <si>
     <t>Notes:</t>
   </si>
@@ -4643,7 +4643,7 @@
                   <c:v>4449</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4524</c:v>
+                  <c:v>4732</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5243,7 +5243,7 @@
                   <c:v>50075</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5319</c:v>
+                  <c:v>5111</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>359266</v>
+        <v>359474</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -6934,7 +6934,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-245</v>
+        <v>-453</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>20270.326666666671</v>
+        <v>20408.993333333328</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>6942.3366666666698</v>
+        <v>6873.0033333333267</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-27212.66333333333</v>
+        <v>-27281.996666666673</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7028,15 +7028,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>158329</v>
+        <v>158537</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>38573.666666666672</v>
+        <v>38712.333333333328</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7044,11 +7044,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>20270.326666666671</v>
+        <v>20408.993333333328</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹20,270</v>
+        <v>Receive ₹20,409</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7062,11 +7062,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>48581.666666666672</v>
+        <v>48512.333333333328</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7074,11 +7074,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>6942.3366666666698</v>
+        <v>6873.0033333333267</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹6,942</v>
+        <v>Receive ₹6,873</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7092,11 +7092,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-87155.333333333328</v>
+        <v>-87224.666666666672</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7104,11 +7104,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-27212.66333333333</v>
+        <v>-27281.996666666673</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹27,213</v>
+        <v>Pay ₹27,282</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46178</v>
+        <v>46179</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>359266</v>
+        <v>359474</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-245</v>
+        <v>-453</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
@@ -7506,7 +7506,7 @@
       </c>
       <c r="B15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A15)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>4524</v>
+        <v>4732</v>
       </c>
       <c r="C15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A15)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>5319</v>
+        <v>5111</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -8868,10 +8868,18 @@
       </c>
     </row>
     <row r="79" spans="1:4" ht="15" customHeight="1">
-      <c r="A79" s="38"/>
-      <c r="B79" s="39"/>
-      <c r="C79" s="40"/>
-      <c r="D79" s="39"/>
+      <c r="A79" s="38">
+        <v>46179</v>
+      </c>
+      <c r="B79" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C79" s="40">
+        <v>208</v>
+      </c>
+      <c r="D79" s="39" t="s">
+        <v>963</v>
+      </c>
     </row>
     <row r="80" spans="1:4" ht="15" customHeight="1">
       <c r="A80" s="35"/>
@@ -34910,15 +34918,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>158329</v>
+        <v>158537</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>38573.666666666672</v>
+        <v>38712.333333333328</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34926,7 +34934,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>38573.666666666672</v>
+        <v>38712.333333333328</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -34934,7 +34942,7 @@
       </c>
       <c r="H8" s="88">
         <f>F8-G8</f>
-        <v>20270.326666666671</v>
+        <v>20408.993333333328</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -34947,11 +34955,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>48581.666666666672</v>
+        <v>48512.333333333328</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34959,7 +34967,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>48581.666666666672</v>
+        <v>48512.333333333328</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -34967,7 +34975,7 @@
       </c>
       <c r="H9" s="89">
         <f>F9-G9</f>
-        <v>6942.3366666666698</v>
+        <v>6873.0033333333267</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -34980,11 +34988,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>119755.33333333333</v>
+        <v>119824.66666666667</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-87155.333333333328</v>
+        <v>-87224.666666666672</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -34992,7 +35000,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-87155.333333333328</v>
+        <v>-87224.666666666672</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -35000,7 +35008,7 @@
       </c>
       <c r="H10" s="88">
         <f>F10-G10</f>
-        <v>-27212.66333333333</v>
+        <v>-27281.996666666673</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="90" customFormat="1" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Latest collection and sales updates
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614187F4-154F-304F-895A-B1C1FB5AEF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3591599D-D810-B648-9807-8BA52475E30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2596" uniqueCount="1042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2713" uniqueCount="1095">
   <si>
     <t>Notes:</t>
   </si>
@@ -2949,20 +2949,6 @@
     <t>Bhavana Meenakshi</t>
   </si>
   <si>
-    <t>Shinoob Cousin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sherin - Maroon/navy blue(1099), Lakshmi - Navy Blue &amp; Maroon, Jaimy - Peacok Blue/Maroon, Shinoob Cousin - Lavender/Violet and Purple/Green </t>
-  </si>
-  <si>
-    <t>Peacok Blue/Maroon - 2
-Navy Blue/Maroon - 2
-Grey/Blue - 1</t>
-  </si>
-  <si>
-    <t>Cotton 2-piece set with blue floral prints-M (CHR-156), Short Kurti(CHR-151)-L, Dusty Rose Salwar(CHR-77)-L, Chanderis Silk Saree(Yellow-CHR-119), Matka - Lavender/Violet &amp; Purple/Green (CHR-174)</t>
-  </si>
-  <si>
     <t>Saida (1400), Binija (1560), Shinoob Cousin(1000)</t>
   </si>
   <si>
@@ -2975,222 +2961,395 @@
     <t>Prema(XXL)- 550, Shinoob cousin(M)-850</t>
   </si>
   <si>
+    <t>CHR-188</t>
+  </si>
+  <si>
+    <t>CHR-189</t>
+  </si>
+  <si>
+    <t>CHR-190</t>
+  </si>
+  <si>
+    <t>CHR-191</t>
+  </si>
+  <si>
+    <t>CHR-192</t>
+  </si>
+  <si>
+    <t>CHR-193</t>
+  </si>
+  <si>
+    <t>CHR-194</t>
+  </si>
+  <si>
+    <t>CHR-195</t>
+  </si>
+  <si>
+    <t>CHR-196</t>
+  </si>
+  <si>
+    <t>CHR-197</t>
+  </si>
+  <si>
+    <t>CHR-198</t>
+  </si>
+  <si>
+    <t>CHR-199</t>
+  </si>
+  <si>
+    <t>CHR-200</t>
+  </si>
+  <si>
+    <t>CHR-201</t>
+  </si>
+  <si>
+    <t>CHR-202</t>
+  </si>
+  <si>
+    <t>CHR-203</t>
+  </si>
+  <si>
+    <t>CHR-204</t>
+  </si>
+  <si>
+    <t>CHR-205</t>
+  </si>
+  <si>
+    <t>CHR-206</t>
+  </si>
+  <si>
+    <t>CHR-207</t>
+  </si>
+  <si>
+    <t>CHR-208</t>
+  </si>
+  <si>
+    <t>CHR-209</t>
+  </si>
+  <si>
+    <t>CHR-210</t>
+  </si>
+  <si>
+    <t>CHR-211</t>
+  </si>
+  <si>
+    <t>CHR-212</t>
+  </si>
+  <si>
+    <t>CHR-213</t>
+  </si>
+  <si>
+    <t>CHR-214</t>
+  </si>
+  <si>
+    <t>CHR-215</t>
+  </si>
+  <si>
+    <t>CHR-216</t>
+  </si>
+  <si>
+    <t>CHR-217</t>
+  </si>
+  <si>
+    <t>CHR-218</t>
+  </si>
+  <si>
+    <t>CHR-219</t>
+  </si>
+  <si>
+    <t>CHR-220</t>
+  </si>
+  <si>
+    <t>CHR-221</t>
+  </si>
+  <si>
+    <t>CHR-222</t>
+  </si>
+  <si>
+    <t>CHR-223</t>
+  </si>
+  <si>
+    <t>CHR-224</t>
+  </si>
+  <si>
+    <t>CHR-225</t>
+  </si>
+  <si>
+    <t>Yellow Lotus Saree Line</t>
+  </si>
+  <si>
+    <t>Postal</t>
+  </si>
+  <si>
+    <t>Temple design preordered - Yet to share the item</t>
+  </si>
+  <si>
+    <t>Banarasil Silk (Chikku Maroon)</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Chikku Green)</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Golden Yellow Green)</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Golden Yellow Blue)</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (New Design)</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (Leaf design)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New </t>
+  </si>
+  <si>
+    <t>Light green/dark green, navy/light, violet/green (leaf designs)</t>
+  </si>
+  <si>
+    <t>rust orange/coffee brown, peacock blue/navy, red/green, mustard/blue, chikku maroon, chikku green, golden yellow &amp; green triangle</t>
+  </si>
+  <si>
+    <t>Green/maroon - Rajitha Teacher</t>
+  </si>
+  <si>
+    <t>Rajitha Teacher</t>
+  </si>
+  <si>
+    <t>Green/maroon banarasi new design</t>
+  </si>
+  <si>
+    <t>Sheeba George</t>
+  </si>
+  <si>
+    <t>Soji Thomas</t>
+  </si>
+  <si>
+    <t>Jessy Joseph</t>
+  </si>
+  <si>
+    <t>Preetha</t>
+  </si>
+  <si>
+    <t>Prasanna</t>
+  </si>
+  <si>
+    <t>Philomina Anto</t>
+  </si>
+  <si>
+    <t>Sanam</t>
+  </si>
+  <si>
+    <t>Geetha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silk Sarees </t>
+  </si>
+  <si>
+    <t>Green/maroon border, maroon peacock blue, light green &amp; bottle green, purple &amp; blue</t>
+  </si>
+  <si>
+    <t>Floral green, floral peach, floral lavender</t>
+  </si>
+  <si>
+    <t>Kerala Sarees with Floral design</t>
+  </si>
+  <si>
+    <t>Kerala Saree with small temple design</t>
+  </si>
+  <si>
+    <t>Small temple design</t>
+  </si>
+  <si>
+    <t>Cotton Saree Collections (Jari Check)</t>
+  </si>
+  <si>
+    <t>Light blue/onion peel, brown/dark maroon, black/light green</t>
+  </si>
+  <si>
+    <t>Cotton Saree Collections (Tower Check)</t>
+  </si>
+  <si>
+    <t>Cotton Saree Collections (Body Jergai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mustard, navy, rani pink, olive green (×2), purple </t>
+  </si>
+  <si>
+    <t>Linen Saree Semi Party Wear Collections</t>
+  </si>
+  <si>
+    <t>Pink, grey, onion peel, blue</t>
+  </si>
+  <si>
+    <t>Kerala Saree Floral Embroidery</t>
+  </si>
+  <si>
+    <t>Floral Embroidery</t>
+  </si>
+  <si>
+    <t>Semi Silk Saree Collections</t>
+  </si>
+  <si>
+    <t>Peach, light blue, pink, light green</t>
+  </si>
+  <si>
+    <t>Tissue Fancy Saree with Butta</t>
+  </si>
+  <si>
+    <t>Navy/blue, green/navy, maroon/grey, red/maroon, dark green/navy</t>
+  </si>
+  <si>
+    <t>Tissue mulmul (soft cotton) blend sarees</t>
+  </si>
+  <si>
+    <t>Tusser Silk Saree Collection</t>
+  </si>
+  <si>
+    <t>Blue, pink, yellow, maroon, deep blue, green</t>
+  </si>
+  <si>
+    <t>Linen Saree</t>
+  </si>
+  <si>
+    <t>Yellow</t>
+  </si>
+  <si>
+    <t>Kalyani Cotton Sarees with check</t>
+  </si>
+  <si>
+    <t>Matka Saree Collections</t>
+  </si>
+  <si>
+    <t>Black/pink, black/orange, violet/bottle green</t>
+  </si>
+  <si>
+    <t>Matka Saree</t>
+  </si>
+  <si>
+    <t>Golden yellow/bottle green</t>
+  </si>
+  <si>
+    <t>Cotton Saree Collection</t>
+  </si>
+  <si>
+    <t>Cotton Saree Collection ( Kabhali Check)</t>
+  </si>
+  <si>
+    <t>Navy/blue, yellow/peacock blue, violet/mustard, turquoise/violet</t>
+  </si>
+  <si>
+    <t>Kerala Saree Collections Check/Floral</t>
+  </si>
+  <si>
+    <t>Checks/floral + leaf, checks/floral + kathakali</t>
+  </si>
+  <si>
+    <t>Cotton Saree with Small and big borders</t>
+  </si>
+  <si>
+    <t>Cotton Lines</t>
+  </si>
+  <si>
+    <t>Maroon/black, violet/red</t>
+  </si>
+  <si>
+    <t>Kerala Saree with lines</t>
+  </si>
+  <si>
+    <t>Jeeja Anil</t>
+  </si>
+  <si>
+    <t>Sumi Boben</t>
+  </si>
+  <si>
+    <t>Jet Black (CHR-119)</t>
+  </si>
+  <si>
+    <t>Jinu Varghese</t>
+  </si>
+  <si>
+    <t>Blue (CHR-119)</t>
+  </si>
+  <si>
+    <t>Smitha S</t>
+  </si>
+  <si>
+    <t>Jayalakshmi, Preetha, Prasanna, Philomina, Smitha S</t>
+  </si>
+  <si>
+    <t>Raji V T</t>
+  </si>
+  <si>
+    <t>Sushama Bhaskar</t>
+  </si>
+  <si>
+    <t>Sanam, Geetha, Unknown, Jessy Joseph, Soji Thomas, Sheeba George, Sushma Bhaskar</t>
+  </si>
+  <si>
+    <t>CHR-194-Light Blue cotton, CHR-206 - green temple/brown</t>
+  </si>
+  <si>
+    <t>Green, pink, navy blue, dark navy, dark maroon, red, orange</t>
+  </si>
+  <si>
+    <t>Denny - Light Blue</t>
+  </si>
+  <si>
+    <t>Grey/black, brown/navy, purple/blue, mustard/blue</t>
+  </si>
+  <si>
+    <t>Denny - green temple/brown</t>
+  </si>
+  <si>
+    <t>Light Majenta - Latha</t>
+  </si>
+  <si>
+    <t>Grey</t>
+  </si>
+  <si>
+    <t>CHR-202 - Yellow Linen(699), CHR-200 - Tissue Mulmul(1250), CHR-206 - Grey/Black &amp; purple/blue</t>
+  </si>
+  <si>
+    <t>Sherin - Maroon/navy blue(1099), Lakshmi - Navy Blue &amp; Maroon, Jaimy - Peacok Blue/Maroon, Shinoob Cousin - Lavender/Violet</t>
+  </si>
+  <si>
+    <t>Peacok Blue/Maroon - 2,
+Navy Blue/Maroon - 2,
+Grey/Blue - 1, Purple/Green - 1</t>
+  </si>
+  <si>
+    <t>red/maroon - Nishitha</t>
+  </si>
+  <si>
+    <t>Nishitha (Shinoob Cousin)</t>
+  </si>
+  <si>
+    <t>Cotton 2-piece set with blue floral prints-M (CHR-156), Short Kurti(CHR-151)-L, Dusty Rose Salwar(CHR-77)-L, Chanderis Silk Saree(Yellow-CHR-119), Matka - Lavender/Violet(CHR-174), red/maroon tissue fancy (CHR-199)</t>
+  </si>
+  <si>
+    <t>Nishitha Friend</t>
+  </si>
+  <si>
+    <t>Blue/maroon, light green/maroon</t>
+  </si>
+  <si>
+    <t>Nishitha Friend - brown/maroon (1100)</t>
+  </si>
+  <si>
+    <t>Orange (CHR-119)</t>
+  </si>
+  <si>
+    <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
+Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned, Sumi Boben (Jet black), Jinu (Blue), Raji VT(Black), Nishitha friend (Orange)</t>
+  </si>
+  <si>
     <t xml:space="preserve">
-Blue (2), Maroon (1), Orange (1), Black(3), White(5)</t>
-  </si>
-  <si>
-    <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
-Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned</t>
-  </si>
-  <si>
-    <t>CHR-188</t>
-  </si>
-  <si>
-    <t>CHR-189</t>
-  </si>
-  <si>
-    <t>CHR-190</t>
-  </si>
-  <si>
-    <t>CHR-191</t>
-  </si>
-  <si>
-    <t>CHR-192</t>
-  </si>
-  <si>
-    <t>CHR-193</t>
-  </si>
-  <si>
-    <t>CHR-194</t>
-  </si>
-  <si>
-    <t>CHR-195</t>
-  </si>
-  <si>
-    <t>CHR-196</t>
-  </si>
-  <si>
-    <t>CHR-197</t>
-  </si>
-  <si>
-    <t>CHR-198</t>
-  </si>
-  <si>
-    <t>CHR-199</t>
-  </si>
-  <si>
-    <t>CHR-200</t>
-  </si>
-  <si>
-    <t>CHR-201</t>
-  </si>
-  <si>
-    <t>CHR-202</t>
-  </si>
-  <si>
-    <t>CHR-203</t>
-  </si>
-  <si>
-    <t>CHR-204</t>
-  </si>
-  <si>
-    <t>CHR-205</t>
-  </si>
-  <si>
-    <t>CHR-206</t>
-  </si>
-  <si>
-    <t>CHR-207</t>
-  </si>
-  <si>
-    <t>CHR-208</t>
-  </si>
-  <si>
-    <t>CHR-209</t>
-  </si>
-  <si>
-    <t>CHR-210</t>
-  </si>
-  <si>
-    <t>CHR-211</t>
-  </si>
-  <si>
-    <t>CHR-212</t>
-  </si>
-  <si>
-    <t>CHR-213</t>
-  </si>
-  <si>
-    <t>CHR-214</t>
-  </si>
-  <si>
-    <t>CHR-215</t>
-  </si>
-  <si>
-    <t>CHR-216</t>
-  </si>
-  <si>
-    <t>CHR-217</t>
-  </si>
-  <si>
-    <t>CHR-218</t>
-  </si>
-  <si>
-    <t>CHR-219</t>
-  </si>
-  <si>
-    <t>CHR-220</t>
-  </si>
-  <si>
-    <t>CHR-221</t>
-  </si>
-  <si>
-    <t>CHR-222</t>
-  </si>
-  <si>
-    <t>CHR-223</t>
-  </si>
-  <si>
-    <t>CHR-224</t>
-  </si>
-  <si>
-    <t>CHR-225</t>
-  </si>
-  <si>
-    <t>Yellow Lotus Saree Line</t>
-  </si>
-  <si>
-    <t>Postal</t>
-  </si>
-  <si>
-    <t>Temple design preordered - Yet to share the item</t>
-  </si>
-  <si>
-    <t>Banarasil Silk (Chikku Maroon)</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Chikku Green)</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Golden Yellow Green)</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Golden Yellow Blue)</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (New Design)</t>
-  </si>
-  <si>
-    <t>Banarasi Silk (Leaf design)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New </t>
-  </si>
-  <si>
-    <t>Light green/dark green, navy/light, violet/green (leaf designs)</t>
-  </si>
-  <si>
-    <t>rust orange/coffee brown, peacock blue/navy, red/green, mustard/blue, chikku maroon, chikku green, golden yellow &amp; green triangle</t>
-  </si>
-  <si>
-    <t>Green/maroon - Rajitha Teacher</t>
-  </si>
-  <si>
-    <t>Jayalakshmi, Preetha, Prasanna, Philomina</t>
-  </si>
-  <si>
-    <t>Sanam, Geetha, Unknown, Jessy Joseph, Soji Thomas, Sheeba George</t>
-  </si>
-  <si>
-    <t>Rajitha Teacher</t>
-  </si>
-  <si>
-    <t>Green/maroon banarasi new design</t>
-  </si>
-  <si>
-    <t>Sheeba George</t>
-  </si>
-  <si>
-    <t>Soji Thomas</t>
-  </si>
-  <si>
-    <t>Jessy Joseph</t>
-  </si>
-  <si>
-    <t>Preetha</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>Prasanna</t>
-  </si>
-  <si>
-    <t>Philomina Anto</t>
-  </si>
-  <si>
-    <t>Sanam</t>
-  </si>
-  <si>
-    <t>Geetha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silk Sarees </t>
-  </si>
-  <si>
-    <t>Green/maroon border, maroon peacock blue, light green &amp; bottle green, purple &amp; blue</t>
-  </si>
-  <si>
-    <t>Floral green, floral peach, floral lavender</t>
-  </si>
-  <si>
-    <t>Kerala Sarees with Floral design</t>
-  </si>
-  <si>
-    <t>Kerala Saree with small temple design</t>
-  </si>
-  <si>
-    <t>Small temple design</t>
+Maroon (1), Black(2), White(5)</t>
+  </si>
+  <si>
+    <t>brown/maroon (CHR-203: 1100), Rust Orange/Coffee Brown (CHR-188)</t>
   </si>
 </sst>
 </file>
@@ -4109,7 +4268,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>225</c:v>
+                  <c:v>234</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>88</c:v>
@@ -4212,7 +4371,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>106</c:v>
+                  <c:v>155</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>60</c:v>
@@ -4545,7 +4704,7 @@
                   <c:v>63190</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76679.463333333319</c:v>
+                  <c:v>117167.19666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5035,7 +5194,7 @@
                   <c:v>54524</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>32953</c:v>
+                  <c:v>47938</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5475,7 +5634,7 @@
                   <c:v>50075</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-65503</c:v>
+                  <c:v>-50518</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5942,10 +6101,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>317</c:v>
+                  <c:v>326</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-656</c:v>
+                  <c:v>-292</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7132,7 +7291,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>383556</v>
+        <v>390893</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7149,7 +7308,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>388466</v>
+        <v>403451</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7166,7 +7325,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-69642</v>
+        <v>-62305</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7378,15 +7537,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>316402</v>
+        <v>323739</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>127877.5704</v>
+        <v>130323.72619999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>188524.4296</v>
+        <v>193415.27380000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7394,11 +7553,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>51214.403599999991</v>
+        <v>56105.247800000012</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹51,214</v>
+        <v>Pay ₹56,105</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7412,11 +7571,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>127800.85919999999</v>
+        <v>130245.54760000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-73176.859199999992</v>
+        <v>-75621.547600000005</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7424,11 +7583,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-1589.8171999999904</v>
+        <v>-4034.5056000000041</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹1,590</v>
+        <v>Receive ₹4,035</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7442,11 +7601,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>127877.5704</v>
+        <v>130323.72619999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-115347.5704</v>
+        <v>-117793.72619999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7454,11 +7613,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-49624.586399999986</v>
+        <v>-52070.742199999979</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹49,625</v>
+        <v>Receive ₹52,071</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7570,7 +7729,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7586,7 +7745,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>383556</v>
+        <v>390893</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7595,14 +7754,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-69642</v>
+        <v>-62305</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>132522.66333333333</v>
+        <v>173010.39666666667</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7654,7 +7813,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7678,7 +7837,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-656</v>
+        <v>-292</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7742,11 +7901,11 @@
       </c>
       <c r="C15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A15)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>32953</v>
+        <v>47938</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>-65503</v>
+        <v>-50518</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -7874,11 +8033,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>106</v>
+        <v>155</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -7905,7 +8064,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>76679.463333333319</v>
+        <v>117167.19666666666</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9180,7 +9339,7 @@
         <v>246</v>
       </c>
       <c r="D84" s="36" t="s">
-        <v>1011</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15" customHeight="1">
@@ -16691,7 +16850,7 @@
         <v>46188</v>
       </c>
       <c r="B216" s="53" t="s">
-        <v>962</v>
+        <v>1086</v>
       </c>
       <c r="C216" s="54">
         <v>5000</v>
@@ -16705,7 +16864,7 @@
       <c r="F216" s="56"/>
       <c r="G216" s="56"/>
       <c r="H216" s="57" t="s">
-        <v>965</v>
+        <v>1087</v>
       </c>
       <c r="I216" s="53" t="s">
         <v>142</v>
@@ -16730,7 +16889,7 @@
       <c r="F217" s="49"/>
       <c r="G217" s="49"/>
       <c r="H217" s="51" t="s">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="I217" s="49" t="s">
         <v>142</v>
@@ -16741,7 +16900,7 @@
         <v>46191</v>
       </c>
       <c r="B218" s="53" t="s">
-        <v>1025</v>
+        <v>1017</v>
       </c>
       <c r="C218" s="54">
         <v>1380</v>
@@ -16755,7 +16914,7 @@
       <c r="F218" s="56"/>
       <c r="G218" s="56"/>
       <c r="H218" s="57" t="s">
-        <v>1026</v>
+        <v>1018</v>
       </c>
       <c r="I218" s="53" t="s">
         <v>142</v>
@@ -16766,7 +16925,7 @@
         <v>46191</v>
       </c>
       <c r="B219" s="49" t="s">
-        <v>1027</v>
+        <v>1019</v>
       </c>
       <c r="C219" s="50">
         <v>1380</v>
@@ -16791,7 +16950,7 @@
         <v>46191</v>
       </c>
       <c r="B220" s="53" t="s">
-        <v>1028</v>
+        <v>1020</v>
       </c>
       <c r="C220" s="54">
         <v>1380</v>
@@ -16841,7 +17000,7 @@
         <v>46191</v>
       </c>
       <c r="B222" s="53" t="s">
-        <v>1029</v>
+        <v>1021</v>
       </c>
       <c r="C222" s="54">
         <v>1380</v>
@@ -16866,7 +17025,7 @@
         <v>46191</v>
       </c>
       <c r="B223" s="49" t="s">
-        <v>1030</v>
+        <v>1022</v>
       </c>
       <c r="C223" s="50">
         <v>1380</v>
@@ -16891,7 +17050,7 @@
         <v>46191</v>
       </c>
       <c r="B224" s="53" t="s">
-        <v>1031</v>
+        <v>1065</v>
       </c>
       <c r="C224" s="54">
         <v>1380</v>
@@ -16916,7 +17075,7 @@
         <v>46192</v>
       </c>
       <c r="B225" s="49" t="s">
-        <v>1032</v>
+        <v>1023</v>
       </c>
       <c r="C225" s="50">
         <v>1380</v>
@@ -16941,7 +17100,7 @@
         <v>46192</v>
       </c>
       <c r="B226" s="53" t="s">
-        <v>1033</v>
+        <v>1024</v>
       </c>
       <c r="C226" s="54">
         <v>1380</v>
@@ -16966,7 +17125,7 @@
         <v>46192</v>
       </c>
       <c r="B227" s="49" t="s">
-        <v>1034</v>
+        <v>1025</v>
       </c>
       <c r="C227" s="50">
         <v>1380</v>
@@ -16991,7 +17150,7 @@
         <v>46192</v>
       </c>
       <c r="B228" s="53" t="s">
-        <v>1035</v>
+        <v>1026</v>
       </c>
       <c r="C228" s="54">
         <v>1380</v>
@@ -17011,104 +17170,218 @@
         <v>142</v>
       </c>
     </row>
-    <row r="229" spans="1:9">
-      <c r="A229" s="48"/>
-      <c r="B229" s="49"/>
-      <c r="C229" s="50"/>
-      <c r="D229" s="49"/>
-      <c r="E229" s="49"/>
+    <row r="229" spans="1:9" ht="14">
+      <c r="A229" s="48">
+        <v>46193</v>
+      </c>
+      <c r="B229" s="49" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C229" s="50">
+        <v>699</v>
+      </c>
+      <c r="D229" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E229" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F229" s="49"/>
       <c r="G229" s="49"/>
-      <c r="H229" s="51"/>
-      <c r="I229" s="49"/>
-    </row>
-    <row r="230" spans="1:9">
-      <c r="A230" s="52"/>
-      <c r="B230" s="53"/>
-      <c r="C230" s="54"/>
-      <c r="D230" s="53"/>
-      <c r="E230" s="53"/>
+      <c r="H229" s="51" t="s">
+        <v>1067</v>
+      </c>
+      <c r="I229" s="49" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" ht="14">
+      <c r="A230" s="52">
+        <v>46193</v>
+      </c>
+      <c r="B230" s="53" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C230" s="54">
+        <v>699</v>
+      </c>
+      <c r="D230" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E230" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F230" s="56"/>
       <c r="G230" s="56"/>
-      <c r="H230" s="57"/>
-      <c r="I230" s="53"/>
-    </row>
-    <row r="231" spans="1:9">
-      <c r="A231" s="48"/>
-      <c r="B231" s="49"/>
-      <c r="C231" s="50"/>
-      <c r="D231" s="49"/>
-      <c r="E231" s="49"/>
+      <c r="H230" s="57" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I230" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" ht="14">
+      <c r="A231" s="48">
+        <v>46193</v>
+      </c>
+      <c r="B231" s="49" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C231" s="50">
+        <v>1380</v>
+      </c>
+      <c r="D231" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E231" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F231" s="49"/>
       <c r="G231" s="49"/>
-      <c r="H231" s="51"/>
-      <c r="I231" s="49"/>
-    </row>
-    <row r="232" spans="1:9">
-      <c r="A232" s="52"/>
-      <c r="B232" s="53"/>
-      <c r="C232" s="54"/>
-      <c r="D232" s="53"/>
-      <c r="E232" s="53"/>
+      <c r="H231" s="51" t="s">
+        <v>359</v>
+      </c>
+      <c r="I231" s="49" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" ht="14">
+      <c r="A232" s="52">
+        <v>46193</v>
+      </c>
+      <c r="B232" s="53" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C232" s="54">
+        <v>699</v>
+      </c>
+      <c r="D232" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E232" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F232" s="56"/>
       <c r="G232" s="56"/>
-      <c r="H232" s="57"/>
-      <c r="I232" s="53"/>
-    </row>
-    <row r="233" spans="1:9">
-      <c r="A233" s="48"/>
-      <c r="B233" s="49"/>
-      <c r="C233" s="50"/>
-      <c r="D233" s="49"/>
-      <c r="E233" s="49"/>
+      <c r="H232" s="57" t="s">
+        <v>1067</v>
+      </c>
+      <c r="I232" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" ht="14">
+      <c r="A233" s="48">
+        <v>46193</v>
+      </c>
+      <c r="B233" s="49" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C233" s="50">
+        <v>1380</v>
+      </c>
+      <c r="D233" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E233" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F233" s="49"/>
       <c r="G233" s="49"/>
-      <c r="H233" s="51"/>
-      <c r="I233" s="49"/>
-    </row>
-    <row r="234" spans="1:9">
-      <c r="A234" s="52"/>
-      <c r="B234" s="53"/>
-      <c r="C234" s="54"/>
+      <c r="H233" s="51" t="s">
+        <v>358</v>
+      </c>
+      <c r="I233" s="49" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" ht="14">
+      <c r="A234" s="52">
+        <v>46193</v>
+      </c>
+      <c r="B234" s="53" t="s">
+        <v>161</v>
+      </c>
+      <c r="C234" s="54">
+        <v>2500</v>
+      </c>
       <c r="D234" s="53"/>
       <c r="E234" s="53"/>
       <c r="F234" s="56"/>
       <c r="G234" s="56"/>
-      <c r="H234" s="57"/>
-      <c r="I234" s="53"/>
-    </row>
-    <row r="235" spans="1:9">
-      <c r="A235" s="48"/>
-      <c r="B235" s="49"/>
-      <c r="C235" s="50"/>
+      <c r="H234" s="57" t="s">
+        <v>1075</v>
+      </c>
+      <c r="I234" s="53" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" ht="28">
+      <c r="A235" s="48">
+        <v>46193</v>
+      </c>
+      <c r="B235" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="C235" s="50">
+        <v>4449</v>
+      </c>
       <c r="D235" s="49"/>
       <c r="E235" s="49"/>
       <c r="F235" s="49"/>
       <c r="G235" s="49"/>
-      <c r="H235" s="51"/>
-      <c r="I235" s="49"/>
-    </row>
-    <row r="236" spans="1:9">
-      <c r="A236" s="52"/>
-      <c r="B236" s="53"/>
-      <c r="C236" s="54"/>
+      <c r="H235" s="51" t="s">
+        <v>1082</v>
+      </c>
+      <c r="I235" s="49" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" ht="14">
+      <c r="A236" s="52">
+        <v>46194</v>
+      </c>
+      <c r="B236" s="53" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C236" s="54">
+        <v>699</v>
+      </c>
       <c r="D236" s="53"/>
       <c r="E236" s="53"/>
       <c r="F236" s="56"/>
       <c r="G236" s="56"/>
-      <c r="H236" s="57"/>
-      <c r="I236" s="53"/>
-    </row>
-    <row r="237" spans="1:9">
-      <c r="A237" s="48"/>
-      <c r="B237" s="49"/>
-      <c r="C237" s="50"/>
-      <c r="D237" s="49"/>
-      <c r="E237" s="49"/>
+      <c r="H236" s="57" t="s">
+        <v>1091</v>
+      </c>
+      <c r="I236" s="53" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" ht="28">
+      <c r="A237" s="48">
+        <v>46194</v>
+      </c>
+      <c r="B237" s="49" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C237" s="50">
+        <v>2480</v>
+      </c>
+      <c r="D237" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E237" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F237" s="49"/>
       <c r="G237" s="49"/>
-      <c r="H237" s="51"/>
-      <c r="I237" s="49"/>
+      <c r="H237" s="51" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I237" s="49" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="238" spans="1:9">
       <c r="A238" s="52"/>
@@ -24996,7 +25269,7 @@
         <v>1075</v>
       </c>
       <c r="L78" s="66" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="M78" s="66"/>
       <c r="N78" s="66" t="s">
@@ -27187,7 +27460,7 @@
       <c r="S119" s="69"/>
       <c r="T119" s="69"/>
     </row>
-    <row r="120" spans="1:246" ht="158" customHeight="1">
+    <row r="120" spans="1:246" ht="175" customHeight="1">
       <c r="A120" s="66" t="s">
         <v>703</v>
       </c>
@@ -27204,14 +27477,14 @@
         <v>699</v>
       </c>
       <c r="F120" s="67">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G120" s="67">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H120" s="66">
         <f t="shared" si="9"/>
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I120" s="66">
         <f>IF(D120&lt;&gt;"",D120,IFERROR(E120/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -27219,14 +27492,14 @@
       </c>
       <c r="J120" s="66">
         <f t="shared" si="10"/>
-        <v>15082.319999999987</v>
+        <v>15920.226666666653</v>
       </c>
       <c r="K120" s="66">
         <f t="shared" si="11"/>
-        <v>5446.3933333333289</v>
+        <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="66" t="s">
-        <v>971</v>
+        <v>1092</v>
       </c>
       <c r="M120" s="66" t="s">
         <v>49</v>
@@ -27236,7 +27509,7 @@
       </c>
       <c r="O120" s="66"/>
       <c r="P120" s="66" t="s">
-        <v>970</v>
+        <v>1093</v>
       </c>
       <c r="Q120" s="66"/>
       <c r="R120" s="66"/>
@@ -29580,14 +29853,14 @@
         <v>590</v>
       </c>
       <c r="L152" s="66" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="M152" s="66"/>
       <c r="N152" s="66" t="s">
         <v>510</v>
       </c>
       <c r="O152" s="66" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="P152" s="66" t="s">
         <v>792</v>
@@ -29850,7 +30123,7 @@
         <v>1050</v>
       </c>
       <c r="L157" s="69" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="M157" s="69"/>
       <c r="N157" s="69" t="s">
@@ -30778,10 +31051,10 @@
         <v>1250</v>
       </c>
       <c r="F175" s="79">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G175" s="79">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H175" s="78">
         <f t="shared" si="15"/>
@@ -30793,14 +31066,14 @@
       </c>
       <c r="J175" s="78">
         <f t="shared" si="16"/>
-        <v>3491.25</v>
+        <v>2793</v>
       </c>
       <c r="K175" s="78">
         <f t="shared" si="17"/>
-        <v>3491.25</v>
+        <v>4189.5</v>
       </c>
       <c r="L175" s="69" t="s">
-        <v>963</v>
+        <v>1083</v>
       </c>
       <c r="M175" s="69"/>
       <c r="N175" s="69" t="s">
@@ -30808,7 +31081,7 @@
       </c>
       <c r="O175" s="69"/>
       <c r="P175" s="69" t="s">
-        <v>964</v>
+        <v>1084</v>
       </c>
       <c r="Q175" s="69"/>
       <c r="R175" s="69"/>
@@ -31192,7 +31465,7 @@
         <v>876</v>
       </c>
       <c r="B183" s="69" t="s">
-        <v>1010</v>
+        <v>1004</v>
       </c>
       <c r="C183" s="69" t="s">
         <v>95</v>
@@ -31241,7 +31514,7 @@
         <v>877</v>
       </c>
       <c r="B184" s="66" t="s">
-        <v>1013</v>
+        <v>1007</v>
       </c>
       <c r="C184" s="66" t="s">
         <v>95</v>
@@ -31253,10 +31526,10 @@
         <v>1380</v>
       </c>
       <c r="F184" s="81">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G184" s="81">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H184" s="80">
         <f t="shared" ref="H184:H226" si="23">F184+IF(LEN(G184)=0,0,G184)</f>
@@ -31268,14 +31541,14 @@
       </c>
       <c r="J184" s="80">
         <f t="shared" si="21"/>
-        <v>5346</v>
+        <v>6237</v>
       </c>
       <c r="K184" s="80">
         <f t="shared" si="22"/>
-        <v>12474</v>
+        <v>11583</v>
       </c>
       <c r="L184" s="66" t="s">
-        <v>1024</v>
+        <v>1074</v>
       </c>
       <c r="M184" s="66"/>
       <c r="N184" s="66" t="s">
@@ -31293,7 +31566,7 @@
         <v>878</v>
       </c>
       <c r="B185" s="69" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="C185" s="69" t="s">
         <v>95</v>
@@ -31305,10 +31578,10 @@
         <v>1380</v>
       </c>
       <c r="F185" s="79">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G185" s="79">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H185" s="78">
         <f t="shared" si="23"/>
@@ -31320,18 +31593,18 @@
       </c>
       <c r="J185" s="78">
         <f t="shared" si="21"/>
-        <v>3564</v>
+        <v>4455</v>
       </c>
       <c r="K185" s="78">
         <f t="shared" si="22"/>
-        <v>891</v>
+        <v>0</v>
       </c>
       <c r="L185" s="69" t="s">
-        <v>1023</v>
+        <v>1071</v>
       </c>
       <c r="M185" s="69"/>
       <c r="N185" s="69" t="s">
-        <v>510</v>
+        <v>425</v>
       </c>
       <c r="O185" s="69"/>
       <c r="P185" s="69"/>
@@ -31395,7 +31668,7 @@
         <v>880</v>
       </c>
       <c r="B187" s="69" t="s">
-        <v>1015</v>
+        <v>1009</v>
       </c>
       <c r="C187" s="69" t="s">
         <v>95</v>
@@ -31445,7 +31718,7 @@
         <v>881</v>
       </c>
       <c r="B188" s="66" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
       <c r="C188" s="66" t="s">
         <v>95</v>
@@ -31492,10 +31765,10 @@
     </row>
     <row r="189" spans="1:20" ht="45">
       <c r="A189" s="69" t="s">
-        <v>972</v>
+        <v>966</v>
       </c>
       <c r="B189" s="66" t="s">
-        <v>1017</v>
+        <v>1011</v>
       </c>
       <c r="C189" s="66" t="s">
         <v>95</v>
@@ -31529,7 +31802,7 @@
         <v>6237</v>
       </c>
       <c r="L189" s="69" t="s">
-        <v>1022</v>
+        <v>1016</v>
       </c>
       <c r="M189" s="69"/>
       <c r="N189" s="69" t="s">
@@ -31537,7 +31810,7 @@
       </c>
       <c r="O189" s="69"/>
       <c r="P189" s="69" t="s">
-        <v>1021</v>
+        <v>1015</v>
       </c>
       <c r="Q189" s="69"/>
       <c r="R189" s="69"/>
@@ -31546,10 +31819,10 @@
     </row>
     <row r="190" spans="1:20" ht="15">
       <c r="A190" s="66" t="s">
-        <v>973</v>
+        <v>967</v>
       </c>
       <c r="B190" s="69" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="C190" s="69" t="s">
         <v>95</v>
@@ -31585,20 +31858,20 @@
       <c r="L190" s="66"/>
       <c r="M190" s="66"/>
       <c r="N190" s="61" t="s">
-        <v>1019</v>
+        <v>1013</v>
       </c>
       <c r="P190" s="61" t="s">
-        <v>1020</v>
+        <v>1014</v>
       </c>
       <c r="S190" s="61"/>
       <c r="T190" s="61"/>
     </row>
     <row r="191" spans="1:20" ht="30">
       <c r="A191" s="69" t="s">
-        <v>974</v>
+        <v>968</v>
       </c>
       <c r="B191" s="66" t="s">
-        <v>1036</v>
+        <v>1027</v>
       </c>
       <c r="C191" s="66" t="s">
         <v>95</v>
@@ -31637,17 +31910,17 @@
         <v>598</v>
       </c>
       <c r="P191" s="61" t="s">
-        <v>1037</v>
+        <v>1028</v>
       </c>
       <c r="S191" s="61"/>
       <c r="T191" s="61"/>
     </row>
     <row r="192" spans="1:20" ht="15">
       <c r="A192" s="66" t="s">
-        <v>975</v>
+        <v>969</v>
       </c>
       <c r="B192" s="69" t="s">
-        <v>1039</v>
+        <v>1030</v>
       </c>
       <c r="C192" s="69" t="s">
         <v>95</v>
@@ -31686,17 +31959,17 @@
         <v>598</v>
       </c>
       <c r="P192" s="61" t="s">
-        <v>1038</v>
+        <v>1029</v>
       </c>
       <c r="S192" s="61"/>
       <c r="T192" s="61"/>
     </row>
     <row r="193" spans="1:20" ht="15">
       <c r="A193" s="69" t="s">
-        <v>976</v>
+        <v>970</v>
       </c>
       <c r="B193" s="66" t="s">
-        <v>1040</v>
+        <v>1031</v>
       </c>
       <c r="C193" s="66" t="s">
         <v>95</v>
@@ -31735,32 +32008,40 @@
         <v>598</v>
       </c>
       <c r="P193" s="61" t="s">
-        <v>1041</v>
+        <v>1032</v>
       </c>
       <c r="S193" s="61"/>
       <c r="T193" s="61"/>
     </row>
     <row r="194" spans="1:20" ht="15">
       <c r="A194" s="66" t="s">
-        <v>977</v>
-      </c>
-      <c r="B194" s="66"/>
-      <c r="C194" s="66"/>
-      <c r="D194" s="67"/>
-      <c r="E194" s="67"/>
+        <v>971</v>
+      </c>
+      <c r="B194" s="66" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C194" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D194" s="67">
+        <v>790</v>
+      </c>
+      <c r="E194" s="67">
+        <v>1250</v>
+      </c>
       <c r="F194" s="81">
         <v>0</v>
       </c>
       <c r="G194" s="81">
-        <v>-9</v>
+        <v>3</v>
       </c>
       <c r="H194" s="80">
         <f t="shared" si="23"/>
-        <v>-9</v>
+        <v>3</v>
       </c>
       <c r="I194" s="80">
         <f>IF(D194&lt;&gt;"",D194,IFERROR(E194/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>790</v>
       </c>
       <c r="J194" s="80">
         <f t="shared" si="21"/>
@@ -31768,69 +32049,99 @@
       </c>
       <c r="K194" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>2370</v>
       </c>
       <c r="L194" s="66"/>
       <c r="M194" s="66"/>
+      <c r="N194" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P194" s="61" t="s">
+        <v>1034</v>
+      </c>
       <c r="S194" s="61"/>
       <c r="T194" s="61"/>
     </row>
     <row r="195" spans="1:20" ht="15">
       <c r="A195" s="69" t="s">
-        <v>978</v>
-      </c>
-      <c r="B195" s="69"/>
-      <c r="C195" s="69"/>
-      <c r="D195" s="70"/>
-      <c r="E195" s="70"/>
+        <v>972</v>
+      </c>
+      <c r="B195" s="69" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C195" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D195" s="70">
+        <v>781</v>
+      </c>
+      <c r="E195" s="70">
+        <v>1250</v>
+      </c>
       <c r="F195" s="79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G195" s="79">
-        <v>-10</v>
+        <v>7</v>
       </c>
       <c r="H195" s="78">
         <f t="shared" si="23"/>
-        <v>-10</v>
+        <v>8</v>
       </c>
       <c r="I195" s="78">
         <f>IF(D195&lt;&gt;"",D195,IFERROR(E195/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>781</v>
       </c>
       <c r="J195" s="78">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>781</v>
       </c>
       <c r="K195" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L195" s="69"/>
+        <v>5467</v>
+      </c>
+      <c r="L195" s="69" t="s">
+        <v>1077</v>
+      </c>
       <c r="M195" s="69"/>
+      <c r="N195" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P195" s="61" t="s">
+        <v>1076</v>
+      </c>
       <c r="S195" s="61"/>
       <c r="T195" s="61"/>
     </row>
     <row r="196" spans="1:20" ht="15">
       <c r="A196" s="66" t="s">
-        <v>979</v>
-      </c>
-      <c r="B196" s="66"/>
-      <c r="C196" s="66"/>
-      <c r="D196" s="67"/>
-      <c r="E196" s="67"/>
+        <v>973</v>
+      </c>
+      <c r="B196" s="66" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C196" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D196" s="67">
+        <v>797</v>
+      </c>
+      <c r="E196" s="67">
+        <v>1250</v>
+      </c>
       <c r="F196" s="81">
         <v>0</v>
       </c>
       <c r="G196" s="81">
-        <v>-11</v>
+        <v>6</v>
       </c>
       <c r="H196" s="80">
         <f t="shared" si="23"/>
-        <v>-11</v>
+        <v>6</v>
       </c>
       <c r="I196" s="80">
         <f>IF(D196&lt;&gt;"",D196,IFERROR(E196/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>797</v>
       </c>
       <c r="J196" s="80">
         <f t="shared" si="21"/>
@@ -31838,34 +32149,48 @@
       </c>
       <c r="K196" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>4782</v>
       </c>
       <c r="L196" s="66"/>
       <c r="M196" s="66"/>
+      <c r="N196" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P196" s="61" t="s">
+        <v>1037</v>
+      </c>
       <c r="S196" s="61"/>
       <c r="T196" s="61"/>
     </row>
     <row r="197" spans="1:20" ht="15">
       <c r="A197" s="69" t="s">
-        <v>980</v>
-      </c>
-      <c r="B197" s="69"/>
-      <c r="C197" s="69"/>
-      <c r="D197" s="70"/>
-      <c r="E197" s="70"/>
+        <v>974</v>
+      </c>
+      <c r="B197" s="69" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C197" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D197" s="70">
+        <v>772</v>
+      </c>
+      <c r="E197" s="70">
+        <v>1250</v>
+      </c>
       <c r="F197" s="79">
         <v>0</v>
       </c>
       <c r="G197" s="79">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="H197" s="78">
         <f t="shared" si="23"/>
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="I197" s="78">
         <f>IF(D197&lt;&gt;"",D197,IFERROR(E197/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>772</v>
       </c>
       <c r="J197" s="78">
         <f t="shared" si="21"/>
@@ -31873,34 +32198,48 @@
       </c>
       <c r="K197" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>3088</v>
       </c>
       <c r="L197" s="69"/>
       <c r="M197" s="69"/>
+      <c r="N197" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P197" s="61" t="s">
+        <v>1039</v>
+      </c>
       <c r="S197" s="61"/>
       <c r="T197" s="61"/>
     </row>
     <row r="198" spans="1:20" ht="15">
       <c r="A198" s="66" t="s">
-        <v>981</v>
-      </c>
-      <c r="B198" s="66"/>
-      <c r="C198" s="66"/>
-      <c r="D198" s="67"/>
-      <c r="E198" s="67"/>
+        <v>975</v>
+      </c>
+      <c r="B198" s="66" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C198" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D198" s="67">
+        <v>772</v>
+      </c>
+      <c r="E198" s="67">
+        <v>1250</v>
+      </c>
       <c r="F198" s="81">
         <v>0</v>
       </c>
       <c r="G198" s="81">
-        <v>-13</v>
+        <v>1</v>
       </c>
       <c r="H198" s="80">
         <f t="shared" si="23"/>
-        <v>-13</v>
+        <v>1</v>
       </c>
       <c r="I198" s="80">
         <f>IF(D198&lt;&gt;"",D198,IFERROR(E198/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>772</v>
       </c>
       <c r="J198" s="80">
         <f t="shared" si="21"/>
@@ -31908,34 +32247,48 @@
       </c>
       <c r="K198" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>772</v>
       </c>
       <c r="L198" s="66"/>
       <c r="M198" s="66"/>
+      <c r="N198" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P198" s="61" t="s">
+        <v>1041</v>
+      </c>
       <c r="S198" s="61"/>
       <c r="T198" s="61"/>
     </row>
     <row r="199" spans="1:20" ht="15">
       <c r="A199" s="69" t="s">
-        <v>982</v>
-      </c>
-      <c r="B199" s="66"/>
-      <c r="C199" s="66"/>
-      <c r="D199" s="67"/>
-      <c r="E199" s="67"/>
+        <v>976</v>
+      </c>
+      <c r="B199" s="66" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C199" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D199" s="67">
+        <v>467</v>
+      </c>
+      <c r="E199" s="67">
+        <v>850</v>
+      </c>
       <c r="F199" s="79">
         <v>0</v>
       </c>
       <c r="G199" s="79">
-        <v>-14</v>
+        <v>4</v>
       </c>
       <c r="H199" s="78">
         <f t="shared" si="23"/>
-        <v>-14</v>
+        <v>4</v>
       </c>
       <c r="I199" s="78">
         <f>IF(D199&lt;&gt;"",D199,IFERROR(E199/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>467</v>
       </c>
       <c r="J199" s="78">
         <f t="shared" si="21"/>
@@ -31943,104 +32296,150 @@
       </c>
       <c r="K199" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>1868</v>
       </c>
       <c r="L199" s="69"/>
       <c r="M199" s="69"/>
+      <c r="N199" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P199" s="61" t="s">
+        <v>1043</v>
+      </c>
       <c r="S199" s="61"/>
       <c r="T199" s="61"/>
     </row>
-    <row r="200" spans="1:20" ht="15">
+    <row r="200" spans="1:20" ht="30">
       <c r="A200" s="66" t="s">
-        <v>983</v>
-      </c>
-      <c r="B200" s="69"/>
-      <c r="C200" s="69"/>
-      <c r="D200" s="70"/>
-      <c r="E200" s="70"/>
+        <v>977</v>
+      </c>
+      <c r="B200" s="69" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C200" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D200" s="70">
+        <v>866</v>
+      </c>
+      <c r="E200" s="70">
+        <v>1350</v>
+      </c>
       <c r="F200" s="81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G200" s="81">
-        <v>-15</v>
+        <v>4</v>
       </c>
       <c r="H200" s="80">
         <f t="shared" si="23"/>
-        <v>-15</v>
+        <v>5</v>
       </c>
       <c r="I200" s="80">
         <f>IF(D200&lt;&gt;"",D200,IFERROR(E200/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>866</v>
       </c>
       <c r="J200" s="80">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>866</v>
       </c>
       <c r="K200" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L200" s="66"/>
+        <v>3464</v>
+      </c>
+      <c r="L200" s="66" t="s">
+        <v>1085</v>
+      </c>
       <c r="M200" s="66"/>
+      <c r="N200" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P200" s="61" t="s">
+        <v>1045</v>
+      </c>
       <c r="S200" s="61"/>
       <c r="T200" s="61"/>
     </row>
     <row r="201" spans="1:20" ht="15">
       <c r="A201" s="69" t="s">
-        <v>984</v>
-      </c>
-      <c r="B201" s="66"/>
-      <c r="C201" s="66"/>
-      <c r="D201" s="67"/>
-      <c r="E201" s="67"/>
+        <v>978</v>
+      </c>
+      <c r="B201" s="66" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C201" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D201" s="67">
+        <v>724</v>
+      </c>
+      <c r="E201" s="67">
+        <v>1250</v>
+      </c>
       <c r="F201" s="79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G201" s="79">
-        <v>-16</v>
+        <v>1</v>
       </c>
       <c r="H201" s="78">
         <f t="shared" si="23"/>
-        <v>-16</v>
+        <v>2</v>
       </c>
       <c r="I201" s="78">
         <f>IF(D201&lt;&gt;"",D201,IFERROR(E201/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>724</v>
       </c>
       <c r="J201" s="78">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>724</v>
       </c>
       <c r="K201" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L201" s="69"/>
+        <v>724</v>
+      </c>
+      <c r="L201" s="69" t="s">
+        <v>1080</v>
+      </c>
       <c r="M201" s="69"/>
+      <c r="N201" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P201" s="61" t="s">
+        <v>1081</v>
+      </c>
       <c r="S201" s="61"/>
       <c r="T201" s="61"/>
     </row>
     <row r="202" spans="1:20" ht="15">
       <c r="A202" s="66" t="s">
-        <v>985</v>
-      </c>
-      <c r="B202" s="69"/>
-      <c r="C202" s="69"/>
-      <c r="D202" s="70"/>
-      <c r="E202" s="70"/>
+        <v>979</v>
+      </c>
+      <c r="B202" s="69" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C202" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D202" s="70">
+        <v>940</v>
+      </c>
+      <c r="E202" s="70">
+        <v>1500</v>
+      </c>
       <c r="F202" s="81">
         <v>0</v>
       </c>
       <c r="G202" s="81">
-        <v>-17</v>
+        <v>5</v>
       </c>
       <c r="H202" s="80">
         <f t="shared" si="23"/>
-        <v>-17</v>
+        <v>5</v>
       </c>
       <c r="I202" s="80">
         <f>IF(D202&lt;&gt;"",D202,IFERROR(E202/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>940</v>
       </c>
       <c r="J202" s="80">
         <f t="shared" si="21"/>
@@ -32048,104 +32447,150 @@
       </c>
       <c r="K202" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="L202" s="66"/>
       <c r="M202" s="66"/>
+      <c r="N202" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P202" s="61" t="s">
+        <v>1048</v>
+      </c>
       <c r="S202" s="61"/>
       <c r="T202" s="61"/>
     </row>
     <row r="203" spans="1:20" ht="15">
       <c r="A203" s="69" t="s">
-        <v>986</v>
-      </c>
-      <c r="B203" s="66"/>
-      <c r="C203" s="66"/>
-      <c r="D203" s="67"/>
-      <c r="E203" s="67"/>
+        <v>980</v>
+      </c>
+      <c r="B203" s="66" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C203" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D203" s="67">
+        <v>488.25</v>
+      </c>
+      <c r="E203" s="67">
+        <v>699</v>
+      </c>
       <c r="F203" s="79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G203" s="79">
-        <v>-18</v>
+        <v>1</v>
       </c>
       <c r="H203" s="78">
         <f t="shared" si="23"/>
-        <v>-18</v>
+        <v>2</v>
       </c>
       <c r="I203" s="78">
         <f>IF(D203&lt;&gt;"",D203,IFERROR(E203/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>488.25</v>
       </c>
       <c r="J203" s="78">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>488.25</v>
       </c>
       <c r="K203" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L203" s="69"/>
+        <v>488.25</v>
+      </c>
+      <c r="L203" s="69" t="s">
+        <v>147</v>
+      </c>
       <c r="M203" s="69"/>
+      <c r="N203" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P203" s="61" t="s">
+        <v>1050</v>
+      </c>
       <c r="S203" s="61"/>
       <c r="T203" s="61"/>
     </row>
     <row r="204" spans="1:20" ht="15">
       <c r="A204" s="66" t="s">
-        <v>987</v>
-      </c>
-      <c r="B204" s="66"/>
-      <c r="C204" s="66"/>
-      <c r="D204" s="67"/>
-      <c r="E204" s="67"/>
+        <v>981</v>
+      </c>
+      <c r="B204" s="66" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C204" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D204" s="67">
+        <v>880</v>
+      </c>
+      <c r="E204" s="67">
+        <v>1350</v>
+      </c>
       <c r="F204" s="81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G204" s="81">
-        <v>-19</v>
+        <v>2</v>
       </c>
       <c r="H204" s="80">
         <f t="shared" si="23"/>
-        <v>-19</v>
+        <v>3</v>
       </c>
       <c r="I204" s="80">
         <f>IF(D204&lt;&gt;"",D204,IFERROR(E204/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="J204" s="80">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="K204" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L204" s="66"/>
+        <v>1760</v>
+      </c>
+      <c r="L204" s="66" t="s">
+        <v>1090</v>
+      </c>
       <c r="M204" s="66"/>
+      <c r="N204" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P204" s="61" t="s">
+        <v>1089</v>
+      </c>
       <c r="S204" s="61"/>
       <c r="T204" s="61"/>
     </row>
     <row r="205" spans="1:20" ht="15">
       <c r="A205" s="69" t="s">
-        <v>988</v>
-      </c>
-      <c r="B205" s="69"/>
-      <c r="C205" s="69"/>
-      <c r="D205" s="70"/>
-      <c r="E205" s="70"/>
+        <v>982</v>
+      </c>
+      <c r="B205" s="69" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C205" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D205" s="70">
+        <v>761</v>
+      </c>
+      <c r="E205" s="70">
+        <v>1250</v>
+      </c>
       <c r="F205" s="79">
         <v>0</v>
       </c>
       <c r="G205" s="79">
-        <v>-20</v>
+        <v>3</v>
       </c>
       <c r="H205" s="78">
         <f t="shared" si="23"/>
-        <v>-20</v>
+        <v>3</v>
       </c>
       <c r="I205" s="78">
         <f>IF(D205&lt;&gt;"",D205,IFERROR(E205/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="J205" s="78">
         <f t="shared" si="21"/>
@@ -32153,34 +32598,48 @@
       </c>
       <c r="K205" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>2283</v>
       </c>
       <c r="L205" s="69"/>
       <c r="M205" s="69"/>
+      <c r="N205" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P205" s="61" t="s">
+        <v>1053</v>
+      </c>
       <c r="S205" s="61"/>
       <c r="T205" s="61"/>
     </row>
     <row r="206" spans="1:20" ht="15">
       <c r="A206" s="66" t="s">
-        <v>989</v>
-      </c>
-      <c r="B206" s="66"/>
-      <c r="C206" s="66"/>
-      <c r="D206" s="67"/>
-      <c r="E206" s="67"/>
+        <v>983</v>
+      </c>
+      <c r="B206" s="66" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C206" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D206" s="67">
+        <v>761</v>
+      </c>
+      <c r="E206" s="67">
+        <v>1250</v>
+      </c>
       <c r="F206" s="81">
         <v>0</v>
       </c>
       <c r="G206" s="81">
-        <v>-21</v>
+        <v>1</v>
       </c>
       <c r="H206" s="80">
         <f t="shared" si="23"/>
-        <v>-21</v>
+        <v>1</v>
       </c>
       <c r="I206" s="80">
         <f>IF(D206&lt;&gt;"",D206,IFERROR(E206/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="J206" s="80">
         <f t="shared" si="21"/>
@@ -32188,69 +32647,99 @@
       </c>
       <c r="K206" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="L206" s="66"/>
       <c r="M206" s="66"/>
+      <c r="N206" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P206" s="61" t="s">
+        <v>1055</v>
+      </c>
       <c r="S206" s="61"/>
       <c r="T206" s="61"/>
     </row>
     <row r="207" spans="1:20" ht="15">
       <c r="A207" s="69" t="s">
-        <v>990</v>
-      </c>
-      <c r="B207" s="69"/>
-      <c r="C207" s="69"/>
-      <c r="D207" s="70"/>
-      <c r="E207" s="70"/>
+        <v>984</v>
+      </c>
+      <c r="B207" s="69" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C207" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D207" s="70">
+        <v>828</v>
+      </c>
+      <c r="E207" s="70">
+        <v>1250</v>
+      </c>
       <c r="F207" s="79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G207" s="79">
-        <v>-22</v>
+        <v>4</v>
       </c>
       <c r="H207" s="78">
         <f t="shared" si="23"/>
-        <v>-22</v>
+        <v>5</v>
       </c>
       <c r="I207" s="78">
         <f>IF(D207&lt;&gt;"",D207,IFERROR(E207/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>828</v>
       </c>
       <c r="J207" s="78">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>828</v>
       </c>
       <c r="K207" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="L207" s="69"/>
+        <v>3312</v>
+      </c>
+      <c r="L207" s="69" t="s">
+        <v>1079</v>
+      </c>
       <c r="M207" s="69"/>
+      <c r="N207" s="61" t="s">
+        <v>510</v>
+      </c>
+      <c r="P207" s="61" t="s">
+        <v>1078</v>
+      </c>
       <c r="S207" s="61"/>
       <c r="T207" s="61"/>
     </row>
-    <row r="208" spans="1:20" ht="15">
+    <row r="208" spans="1:20" ht="30">
       <c r="A208" s="66" t="s">
-        <v>991</v>
-      </c>
-      <c r="B208" s="66"/>
-      <c r="C208" s="66"/>
-      <c r="D208" s="67"/>
-      <c r="E208" s="67"/>
+        <v>985</v>
+      </c>
+      <c r="B208" s="66" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C208" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D208" s="67">
+        <v>782</v>
+      </c>
+      <c r="E208" s="67">
+        <v>1250</v>
+      </c>
       <c r="F208" s="81">
         <v>0</v>
       </c>
       <c r="G208" s="81">
-        <v>-23</v>
+        <v>4</v>
       </c>
       <c r="H208" s="80">
         <f t="shared" si="23"/>
-        <v>-23</v>
+        <v>4</v>
       </c>
       <c r="I208" s="80">
         <f>IF(D208&lt;&gt;"",D208,IFERROR(E208/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>782</v>
       </c>
       <c r="J208" s="80">
         <f t="shared" si="21"/>
@@ -32258,34 +32747,48 @@
       </c>
       <c r="K208" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>3128</v>
       </c>
       <c r="L208" s="66"/>
       <c r="M208" s="66"/>
+      <c r="N208" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P208" s="61" t="s">
+        <v>1058</v>
+      </c>
       <c r="S208" s="61"/>
       <c r="T208" s="61"/>
     </row>
     <row r="209" spans="1:20" ht="15">
       <c r="A209" s="69" t="s">
-        <v>992</v>
-      </c>
-      <c r="B209" s="66"/>
-      <c r="C209" s="66"/>
-      <c r="D209" s="67"/>
-      <c r="E209" s="67"/>
+        <v>986</v>
+      </c>
+      <c r="B209" s="66" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C209" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D209" s="67">
+        <v>982</v>
+      </c>
+      <c r="E209" s="67">
+        <v>1550</v>
+      </c>
       <c r="F209" s="79">
         <v>0</v>
       </c>
       <c r="G209" s="79">
-        <v>-24</v>
+        <v>2</v>
       </c>
       <c r="H209" s="78">
         <f t="shared" si="23"/>
-        <v>-24</v>
+        <v>2</v>
       </c>
       <c r="I209" s="78">
         <f>IF(D209&lt;&gt;"",D209,IFERROR(E209/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>982</v>
       </c>
       <c r="J209" s="78">
         <f t="shared" si="21"/>
@@ -32293,34 +32796,48 @@
       </c>
       <c r="K209" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>1964</v>
       </c>
       <c r="L209" s="69"/>
       <c r="M209" s="69"/>
+      <c r="N209" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P209" s="61" t="s">
+        <v>1060</v>
+      </c>
       <c r="S209" s="61"/>
       <c r="T209" s="61"/>
     </row>
     <row r="210" spans="1:20" ht="15">
       <c r="A210" s="66" t="s">
-        <v>993</v>
-      </c>
-      <c r="B210" s="69"/>
-      <c r="C210" s="69"/>
-      <c r="D210" s="70"/>
-      <c r="E210" s="70"/>
+        <v>987</v>
+      </c>
+      <c r="B210" s="69" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C210" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="D210" s="70">
+        <v>891</v>
+      </c>
+      <c r="E210" s="70">
+        <v>1350</v>
+      </c>
       <c r="F210" s="81">
         <v>0</v>
       </c>
       <c r="G210" s="81">
-        <v>-25</v>
+        <v>1</v>
       </c>
       <c r="H210" s="80">
         <f t="shared" si="23"/>
-        <v>-25</v>
+        <v>1</v>
       </c>
       <c r="I210" s="80">
         <f>IF(D210&lt;&gt;"",D210,IFERROR(E210/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>891</v>
       </c>
       <c r="J210" s="80">
         <f t="shared" si="21"/>
@@ -32328,34 +32845,48 @@
       </c>
       <c r="K210" s="80">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>891</v>
       </c>
       <c r="L210" s="66"/>
       <c r="M210" s="66"/>
+      <c r="N210" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P210" s="61" t="s">
+        <v>1062</v>
+      </c>
       <c r="S210" s="61"/>
       <c r="T210" s="61"/>
     </row>
     <row r="211" spans="1:20" ht="15">
       <c r="A211" s="69" t="s">
-        <v>994</v>
-      </c>
-      <c r="B211" s="66"/>
-      <c r="C211" s="66"/>
-      <c r="D211" s="67"/>
-      <c r="E211" s="67"/>
+        <v>988</v>
+      </c>
+      <c r="B211" s="66" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C211" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="D211" s="67">
+        <v>922</v>
+      </c>
+      <c r="E211" s="67">
+        <v>1400</v>
+      </c>
       <c r="F211" s="79">
         <v>0</v>
       </c>
       <c r="G211" s="79">
-        <v>-26</v>
+        <v>2</v>
       </c>
       <c r="H211" s="78">
         <f t="shared" si="23"/>
-        <v>-26</v>
+        <v>2</v>
       </c>
       <c r="I211" s="78">
         <f>IF(D211&lt;&gt;"",D211,IFERROR(E211/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>922</v>
       </c>
       <c r="J211" s="78">
         <f t="shared" si="21"/>
@@ -32363,16 +32894,22 @@
       </c>
       <c r="K211" s="78">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>1844</v>
       </c>
       <c r="L211" s="69"/>
       <c r="M211" s="69"/>
+      <c r="N211" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="P211" s="61" t="s">
+        <v>1063</v>
+      </c>
       <c r="S211" s="61"/>
       <c r="T211" s="61"/>
     </row>
     <row r="212" spans="1:20" ht="15">
       <c r="A212" s="66" t="s">
-        <v>995</v>
+        <v>989</v>
       </c>
       <c r="B212" s="69"/>
       <c r="C212" s="69"/>
@@ -32407,7 +32944,7 @@
     </row>
     <row r="213" spans="1:20" ht="15">
       <c r="A213" s="69" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="B213" s="66"/>
       <c r="C213" s="66"/>
@@ -32442,7 +32979,7 @@
     </row>
     <row r="214" spans="1:20" ht="15">
       <c r="A214" s="66" t="s">
-        <v>997</v>
+        <v>991</v>
       </c>
       <c r="B214" s="66"/>
       <c r="C214" s="66"/>
@@ -32477,7 +33014,7 @@
     </row>
     <row r="215" spans="1:20" ht="15">
       <c r="A215" s="69" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="B215" s="69"/>
       <c r="C215" s="69"/>
@@ -32512,7 +33049,7 @@
     </row>
     <row r="216" spans="1:20" ht="15">
       <c r="A216" s="66" t="s">
-        <v>999</v>
+        <v>993</v>
       </c>
       <c r="B216" s="66"/>
       <c r="C216" s="66"/>
@@ -32547,7 +33084,7 @@
     </row>
     <row r="217" spans="1:20" ht="15">
       <c r="A217" s="69" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="B217" s="69"/>
       <c r="C217" s="69"/>
@@ -32582,7 +33119,7 @@
     </row>
     <row r="218" spans="1:20" ht="15">
       <c r="A218" s="66" t="s">
-        <v>1001</v>
+        <v>995</v>
       </c>
       <c r="B218" s="66"/>
       <c r="C218" s="66"/>
@@ -32617,7 +33154,7 @@
     </row>
     <row r="219" spans="1:20" ht="15">
       <c r="A219" s="69" t="s">
-        <v>1002</v>
+        <v>996</v>
       </c>
       <c r="B219" s="66"/>
       <c r="C219" s="66"/>
@@ -32652,7 +33189,7 @@
     </row>
     <row r="220" spans="1:20" ht="15">
       <c r="A220" s="66" t="s">
-        <v>1003</v>
+        <v>997</v>
       </c>
       <c r="B220" s="69"/>
       <c r="C220" s="69"/>
@@ -32687,7 +33224,7 @@
     </row>
     <row r="221" spans="1:20" ht="15">
       <c r="A221" s="69" t="s">
-        <v>1004</v>
+        <v>998</v>
       </c>
       <c r="B221" s="66"/>
       <c r="C221" s="66"/>
@@ -32722,7 +33259,7 @@
     </row>
     <row r="222" spans="1:20" ht="15">
       <c r="A222" s="66" t="s">
-        <v>1005</v>
+        <v>999</v>
       </c>
       <c r="B222" s="69"/>
       <c r="C222" s="69"/>
@@ -32757,7 +33294,7 @@
     </row>
     <row r="223" spans="1:20" ht="15">
       <c r="A223" s="69" t="s">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="B223" s="66"/>
       <c r="C223" s="66"/>
@@ -32792,7 +33329,7 @@
     </row>
     <row r="224" spans="1:20" ht="15">
       <c r="A224" s="66" t="s">
-        <v>1007</v>
+        <v>1001</v>
       </c>
       <c r="B224" s="66"/>
       <c r="C224" s="66"/>
@@ -32827,7 +33364,7 @@
     </row>
     <row r="225" spans="1:20" ht="15">
       <c r="A225" s="69" t="s">
-        <v>1008</v>
+        <v>1002</v>
       </c>
       <c r="B225" s="69"/>
       <c r="C225" s="69"/>
@@ -32862,7 +33399,7 @@
     </row>
     <row r="226" spans="1:20" ht="15">
       <c r="A226" s="66" t="s">
-        <v>1009</v>
+        <v>1003</v>
       </c>
       <c r="B226" s="66"/>
       <c r="C226" s="66"/>
@@ -37353,7 +37890,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>316402</v>
+        <v>323739</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -37361,11 +37898,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>127877.5704</v>
+        <v>130323.72619999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>188524.4296</v>
+        <v>193415.27380000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37373,7 +37910,7 @@
       </c>
       <c r="G4" s="88">
         <f>E4+F4</f>
-        <v>51214.403599999991</v>
+        <v>56105.247800000012</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -37390,11 +37927,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>127800.85919999999</v>
+        <v>130245.54760000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-73176.859199999992</v>
+        <v>-75621.547600000005</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37402,7 +37939,7 @@
       </c>
       <c r="G5" s="89">
         <f>E5+F5</f>
-        <v>-1589.8171999999904</v>
+        <v>-4034.5056000000041</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -37419,11 +37956,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>127877.5704</v>
+        <v>130323.72619999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-115347.5704</v>
+        <v>-117793.72619999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -37431,7 +37968,7 @@
       </c>
       <c r="G6" s="88">
         <f>E6+F6</f>
-        <v>-49624.586399999986</v>
+        <v>-52070.742199999979</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
Latest Sales 6-24 & 6-25
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jun26.xlsx
+++ b/docs/Chiraath-Summary-Jun26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE98F41-E936-CA46-8B2F-F9D6C20FB277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785E3F12-4497-1348-8408-FA40268A10B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2738" uniqueCount="1105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2768" uniqueCount="1111">
   <si>
     <t>Notes:</t>
   </si>
@@ -3105,12 +3105,6 @@
     <t>Light green/dark green, navy/light, violet/green (leaf designs)</t>
   </si>
   <si>
-    <t>rust orange/coffee brown, peacock blue/navy, red/green, mustard/blue, chikku maroon, chikku green, golden yellow &amp; green triangle</t>
-  </si>
-  <si>
-    <t>Green/maroon - Rajitha Teacher</t>
-  </si>
-  <si>
     <t>Rajitha Teacher</t>
   </si>
   <si>
@@ -3311,15 +3305,9 @@
 Grey/Blue - 1, Purple/Green - 1</t>
   </si>
   <si>
-    <t>Nishitha (Shinoob Cousin)</t>
-  </si>
-  <si>
     <t>Cotton 2-piece set with blue floral prints-M (CHR-156), Short Kurti(CHR-151)-L, Dusty Rose Salwar(CHR-77)-L, Chanderis Silk Saree(Yellow-CHR-119), Matka - Lavender/Violet(CHR-174), red/maroon tissue fancy (CHR-199)</t>
   </si>
   <si>
-    <t>Nishitha Friend</t>
-  </si>
-  <si>
     <t>Blue/maroon, light green/maroon</t>
   </si>
   <si>
@@ -3362,24 +3350,54 @@
     <t>CHR-119 Chanderi Blue</t>
   </si>
   <si>
+    <t>Navya - Black Orange</t>
+  </si>
+  <si>
+    <t>Banarasi CM(CHR-183), Black Orange (CHR-204), CHR-199 - Navy/blue &amp; maroon/grey</t>
+  </si>
+  <si>
+    <t>red/maroon - Nishitha, Navy/blue &amp; maroon/grey - Navya</t>
+  </si>
+  <si>
+    <t>Nishida</t>
+  </si>
+  <si>
+    <t>Divya Jacob</t>
+  </si>
+  <si>
+    <t>Razia Salim</t>
+  </si>
+  <si>
+    <t>Banarasi Silk (New Design) - Chikku Green (CHR-188)</t>
+  </si>
+  <si>
+    <t>rust orange/coffee brown, peacock blue/navy, red/green, mustard/blue, chikku maroon, golden yellow &amp; green triangle</t>
+  </si>
+  <si>
+    <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim</t>
+  </si>
+  <si>
+    <t>Baby Johny</t>
+  </si>
+  <si>
+    <t>2026--06-24</t>
+  </si>
+  <si>
+    <t>Chanderi White (CHR-119)</t>
+  </si>
+  <si>
     <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
-Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned, Sumi Boben (Jet black), Jinu (Blue), Raji VT(Black), Nishitha friend (Orange), Karthika (Blue)</t>
+Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned, Sumi Boben (Jet black), Jinu (Blue), Raji VT(Black), Nishitha friend (Orange), Karthika (Blue), SIndhu (White)</t>
   </si>
   <si>
     <t xml:space="preserve">
-Maroon, Black, White(5)</t>
-  </si>
-  <si>
-    <t>Sanam, Geetha, Unknown, Jessy Joseph, Soji Thomas, Sheeba George, Sushma Bhaskar, Navya</t>
-  </si>
-  <si>
-    <t>Navya - Black Orange</t>
-  </si>
-  <si>
-    <t>Banarasi CM(CHR-183), Black Orange (CHR-204), CHR-199 - Navy/blue &amp; maroon/grey</t>
-  </si>
-  <si>
-    <t>red/maroon - Nishitha, Navy/blue &amp; maroon/grey - Navya</t>
+Maroon, Black, White(4)</t>
+  </si>
+  <si>
+    <t>Jayasree</t>
+  </si>
+  <si>
+    <t>Sanam, Geetha, Unknown, Jessy Joseph, Soji Thomas, Sheeba George, Sushma Bhaskar, Navya, Divya Jacob, Baby Johny, Jayashree</t>
   </si>
 </sst>
 </file>
@@ -4298,7 +4316,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>241</c:v>
+                  <c:v>246</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>88</c:v>
@@ -4401,7 +4419,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>148</c:v>
+                  <c:v>143</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>60</c:v>
@@ -4734,7 +4752,7 @@
                   <c:v>63190</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>111984.49333333333</c:v>
+                  <c:v>108001.54</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5064,7 +5082,7 @@
                   <c:v>4449</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>98456</c:v>
+                  <c:v>98616</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5209,22 +5227,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>45448</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>19089</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>16248</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>54177</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>54524</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>55717</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -5649,22 +5667,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>-1863</c:v>
+                  <c:v>-47311</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13937</c:v>
+                  <c:v>-5152</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-5924</c:v>
+                  <c:v>-22172</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-16825</c:v>
+                  <c:v>-71002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>50075</c:v>
+                  <c:v>-4449</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-42739</c:v>
+                  <c:v>-98616</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -6131,10 +6149,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>333</c:v>
+                  <c:v>338</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-299</c:v>
+                  <c:v>-304</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7291,7 +7309,7 @@
     <col min="4" max="4" width="30.1640625" style="6" customWidth="1"/>
     <col min="5" max="5" width="22.1640625" style="6" customWidth="1"/>
     <col min="6" max="6" width="31.1640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="6" customWidth="1"/>
     <col min="8" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
@@ -7306,7 +7324,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>453560</v>
+        <v>453720</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7321,7 +7339,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>398672</v>
+        <v>408891</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7338,7 +7356,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>411230</v>
+        <v>417000</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7355,7 +7373,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-54888</v>
+        <v>-44829</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7390,7 +7408,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>43132.993333333347</v>
+        <v>43239.66</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7400,7 +7418,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>15511.003333333341</v>
+        <v>15457.669999999998</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7410,7 +7428,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-58643.996666666659</v>
+        <v>-58697.33</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7449,15 +7467,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>212623</v>
+        <v>212783</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>61436.333333333343</v>
+        <v>61543</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7465,11 +7483,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>43132.993333333347</v>
+        <v>43239.66</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹43,133</v>
+        <v>Receive ₹43,240</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7483,11 +7501,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>57150.333333333343</v>
+        <v>57097</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7495,11 +7513,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>15511.003333333341</v>
+        <v>15457.669999999998</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹15,511</v>
+        <v>Receive ₹15,458</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7513,11 +7531,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-118586.66666666666</v>
+        <v>-118640</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7525,11 +7543,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-58643.996666666659</v>
+        <v>-58697.33</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹58,644</v>
+        <v>Pay ₹58,697</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7567,15 +7585,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>331518</v>
+        <v>341737</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>132917.24479999999</v>
+        <v>136324.25939999998</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>198600.75520000001</v>
+        <v>205412.74060000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7583,11 +7601,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>61290.729200000002</v>
+        <v>68102.714600000007</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹61,291</v>
+        <v>Pay ₹68,103</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7601,11 +7619,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>132837.5104</v>
+        <v>136242.48120000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-78213.510399999999</v>
+        <v>-81618.481200000009</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7613,11 +7631,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-6626.4683999999979</v>
+        <v>-10031.439200000008</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹6,626</v>
+        <v>Receive ₹10,031</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7631,11 +7649,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>132917.24479999999</v>
+        <v>136324.25939999998</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-120387.24479999999</v>
+        <v>-123794.25939999998</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7643,11 +7661,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-54664.260799999975</v>
+        <v>-58071.27539999997</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹54,664</v>
+        <v>Receive ₹58,071</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7759,7 +7777,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46196</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7768,14 +7786,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>453560</v>
+        <v>453720</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>398672</v>
+        <v>408891</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7784,14 +7802,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-54888</v>
+        <v>-44829</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>167827.69333333333</v>
+        <v>163844.74</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7832,18 +7850,18 @@
       </c>
       <c r="C10" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A10)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>45448</v>
+        <v>0</v>
       </c>
       <c r="D10" s="21">
         <f t="shared" ref="D10:D21" si="0">C10-B10</f>
-        <v>-1863</v>
+        <v>-47311</v>
       </c>
       <c r="F10" s="25" t="s">
         <v>80</v>
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7856,18 +7874,18 @@
       </c>
       <c r="C11" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A11)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>19089</v>
+        <v>0</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>13937</v>
+        <v>-5152</v>
       </c>
       <c r="F11" s="26" t="s">
         <v>82</v>
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-299</v>
+        <v>-304</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7880,11 +7898,11 @@
       </c>
       <c r="C12" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A12)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>16248</v>
+        <v>0</v>
       </c>
       <c r="D12" s="21">
         <f t="shared" si="0"/>
-        <v>-5924</v>
+        <v>-22172</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1">
@@ -7897,11 +7915,11 @@
       </c>
       <c r="C13" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A13)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>54177</v>
+        <v>0</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>-16825</v>
+        <v>-71002</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
@@ -7914,11 +7932,11 @@
       </c>
       <c r="C14" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A14)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>54524</v>
+        <v>0</v>
       </c>
       <c r="D14" s="21">
         <f t="shared" si="0"/>
-        <v>50075</v>
+        <v>-4449</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1">
@@ -7927,15 +7945,15 @@
       </c>
       <c r="B15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A15)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>98456</v>
+        <v>98616</v>
       </c>
       <c r="C15" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$996,"MMM")=$A15)*(YEAR(Sales!$A$2:$A$996)=$B$7)*Sales!$C$2:$C$996),0)</f>
-        <v>55717</v>
+        <v>0</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>-42739</v>
+        <v>-98616</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -8063,11 +8081,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8094,7 +8112,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>111984.49333333333</v>
+        <v>108001.54</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9397,7 +9415,7 @@
         <v>300</v>
       </c>
       <c r="D86" s="36" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15" customHeight="1">
@@ -9411,14 +9429,22 @@
         <v>62</v>
       </c>
       <c r="D87" s="39" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="15" customHeight="1">
-      <c r="A88" s="35"/>
-      <c r="B88" s="36"/>
-      <c r="C88" s="37"/>
-      <c r="D88" s="36"/>
+      <c r="A88" s="35">
+        <v>46197</v>
+      </c>
+      <c r="B88" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C88" s="37">
+        <v>160</v>
+      </c>
+      <c r="D88" s="36" t="s">
+        <v>1085</v>
+      </c>
     </row>
     <row r="89" spans="1:4" ht="15" customHeight="1">
       <c r="A89" s="38"/>
@@ -16896,7 +16922,7 @@
         <v>46188</v>
       </c>
       <c r="B216" s="53" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="C216" s="54">
         <v>5000</v>
@@ -16910,7 +16936,7 @@
       <c r="F216" s="56"/>
       <c r="G216" s="56"/>
       <c r="H216" s="57" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="I216" s="53" t="s">
         <v>142</v>
@@ -16946,7 +16972,7 @@
         <v>46191</v>
       </c>
       <c r="B218" s="53" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="C218" s="54">
         <v>1380</v>
@@ -16960,7 +16986,7 @@
       <c r="F218" s="56"/>
       <c r="G218" s="56"/>
       <c r="H218" s="57" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="I218" s="53" t="s">
         <v>142</v>
@@ -16971,7 +16997,7 @@
         <v>46191</v>
       </c>
       <c r="B219" s="49" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="C219" s="50">
         <v>1380</v>
@@ -16996,7 +17022,7 @@
         <v>46191</v>
       </c>
       <c r="B220" s="53" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="C220" s="54">
         <v>1380</v>
@@ -17046,7 +17072,7 @@
         <v>46191</v>
       </c>
       <c r="B222" s="53" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="C222" s="54">
         <v>1380</v>
@@ -17071,7 +17097,7 @@
         <v>46191</v>
       </c>
       <c r="B223" s="49" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="C223" s="50">
         <v>1380</v>
@@ -17096,7 +17122,7 @@
         <v>46191</v>
       </c>
       <c r="B224" s="53" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="C224" s="54">
         <v>1380</v>
@@ -17121,7 +17147,7 @@
         <v>46192</v>
       </c>
       <c r="B225" s="49" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="C225" s="50">
         <v>1380</v>
@@ -17146,7 +17172,7 @@
         <v>46192</v>
       </c>
       <c r="B226" s="53" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="C226" s="54">
         <v>1380</v>
@@ -17171,7 +17197,7 @@
         <v>46192</v>
       </c>
       <c r="B227" s="49" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="C227" s="50">
         <v>1380</v>
@@ -17196,7 +17222,7 @@
         <v>46192</v>
       </c>
       <c r="B228" s="53" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="C228" s="54">
         <v>1380</v>
@@ -17221,7 +17247,7 @@
         <v>46193</v>
       </c>
       <c r="B229" s="49" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="C229" s="50">
         <v>699</v>
@@ -17235,7 +17261,7 @@
       <c r="F229" s="49"/>
       <c r="G229" s="49"/>
       <c r="H229" s="51" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="I229" s="49" t="s">
         <v>142</v>
@@ -17246,7 +17272,7 @@
         <v>46193</v>
       </c>
       <c r="B230" s="53" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="C230" s="54">
         <v>699</v>
@@ -17260,7 +17286,7 @@
       <c r="F230" s="56"/>
       <c r="G230" s="56"/>
       <c r="H230" s="57" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="I230" s="53" t="s">
         <v>142</v>
@@ -17271,7 +17297,7 @@
         <v>46193</v>
       </c>
       <c r="B231" s="49" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="C231" s="50">
         <v>1380</v>
@@ -17296,7 +17322,7 @@
         <v>46193</v>
       </c>
       <c r="B232" s="53" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="C232" s="54">
         <v>699</v>
@@ -17310,7 +17336,7 @@
       <c r="F232" s="56"/>
       <c r="G232" s="56"/>
       <c r="H232" s="57" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="I232" s="53" t="s">
         <v>142</v>
@@ -17321,7 +17347,7 @@
         <v>46193</v>
       </c>
       <c r="B233" s="49" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="C233" s="50">
         <v>1380</v>
@@ -17356,7 +17382,7 @@
       <c r="F234" s="56"/>
       <c r="G234" s="56"/>
       <c r="H234" s="57" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="I234" s="53" t="s">
         <v>341</v>
@@ -17370,17 +17396,21 @@
         <v>147</v>
       </c>
       <c r="C235" s="50">
-        <v>4449</v>
-      </c>
-      <c r="D235" s="49"/>
-      <c r="E235" s="49"/>
+        <v>4000</v>
+      </c>
+      <c r="D235" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E235" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F235" s="49"/>
       <c r="G235" s="49"/>
       <c r="H235" s="51" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="I235" s="49" t="s">
-        <v>341</v>
+        <v>142</v>
       </c>
     </row>
     <row r="236" spans="1:9" ht="14">
@@ -17388,7 +17418,7 @@
         <v>46194</v>
       </c>
       <c r="B236" s="53" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="C236" s="54">
         <v>699</v>
@@ -17398,7 +17428,7 @@
       <c r="F236" s="56"/>
       <c r="G236" s="56"/>
       <c r="H236" s="57" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="I236" s="53" t="s">
         <v>341</v>
@@ -17409,7 +17439,7 @@
         <v>46194</v>
       </c>
       <c r="B237" s="49" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="C237" s="50">
         <v>2480</v>
@@ -17423,7 +17453,7 @@
       <c r="F237" s="49"/>
       <c r="G237" s="49"/>
       <c r="H237" s="51" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="I237" s="49" t="s">
         <v>142</v>
@@ -17434,7 +17464,7 @@
         <v>46196</v>
       </c>
       <c r="B238" s="53" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="C238" s="54">
         <v>700</v>
@@ -17448,7 +17478,7 @@
       <c r="F238" s="56"/>
       <c r="G238" s="56"/>
       <c r="H238" s="57" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="I238" s="53" t="s">
         <v>142</v>
@@ -17459,7 +17489,7 @@
         <v>46196</v>
       </c>
       <c r="B239" s="49" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="C239" s="50">
         <v>1380</v>
@@ -17473,7 +17503,7 @@
       <c r="F239" s="49"/>
       <c r="G239" s="49"/>
       <c r="H239" s="51" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="I239" s="49" t="s">
         <v>142</v>
@@ -17484,7 +17514,7 @@
         <v>46196</v>
       </c>
       <c r="B240" s="53" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="C240" s="54">
         <v>699</v>
@@ -17498,7 +17528,7 @@
       <c r="F240" s="56"/>
       <c r="G240" s="56"/>
       <c r="H240" s="57" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="I240" s="53" t="s">
         <v>142</v>
@@ -17523,66 +17553,136 @@
       <c r="F241" s="49"/>
       <c r="G241" s="49"/>
       <c r="H241" s="51" t="s">
-        <v>1103</v>
+        <v>1096</v>
       </c>
       <c r="I241" s="49" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="242" spans="1:9">
-      <c r="A242" s="52"/>
-      <c r="B242" s="53"/>
-      <c r="C242" s="54"/>
-      <c r="D242" s="53"/>
-      <c r="E242" s="53"/>
+    <row r="242" spans="1:9" ht="14">
+      <c r="A242" s="52">
+        <v>46197</v>
+      </c>
+      <c r="B242" s="53" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C242" s="54">
+        <v>1380</v>
+      </c>
+      <c r="D242" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E242" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F242" s="56"/>
       <c r="G242" s="56"/>
-      <c r="H242" s="57"/>
-      <c r="I242" s="53"/>
-    </row>
-    <row r="243" spans="1:9">
-      <c r="A243" s="48"/>
-      <c r="B243" s="49"/>
-      <c r="C243" s="50"/>
-      <c r="D243" s="49"/>
-      <c r="E243" s="49"/>
+      <c r="H242" s="57" t="s">
+        <v>358</v>
+      </c>
+      <c r="I242" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" ht="14">
+      <c r="A243" s="48">
+        <v>46197</v>
+      </c>
+      <c r="B243" s="49" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C243" s="50">
+        <v>1380</v>
+      </c>
+      <c r="D243" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E243" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F243" s="49"/>
       <c r="G243" s="49"/>
-      <c r="H243" s="51"/>
-      <c r="I243" s="49"/>
-    </row>
-    <row r="244" spans="1:9">
-      <c r="A244" s="52"/>
-      <c r="B244" s="53"/>
-      <c r="C244" s="54"/>
-      <c r="D244" s="53"/>
-      <c r="E244" s="53"/>
+      <c r="H243" s="51" t="s">
+        <v>1101</v>
+      </c>
+      <c r="I243" s="49" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" ht="14">
+      <c r="A244" s="52">
+        <v>46197</v>
+      </c>
+      <c r="B244" s="53" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C244" s="54">
+        <v>1380</v>
+      </c>
+      <c r="D244" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E244" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F244" s="56"/>
       <c r="G244" s="56"/>
-      <c r="H244" s="57"/>
-      <c r="I244" s="53"/>
-    </row>
-    <row r="245" spans="1:9">
-      <c r="A245" s="48"/>
-      <c r="B245" s="49"/>
-      <c r="C245" s="50"/>
-      <c r="D245" s="49"/>
-      <c r="E245" s="49"/>
+      <c r="H244" s="57" t="s">
+        <v>358</v>
+      </c>
+      <c r="I244" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" ht="14">
+      <c r="A245" s="48" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B245" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="C245" s="50">
+        <v>699</v>
+      </c>
+      <c r="D245" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E245" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F245" s="49"/>
       <c r="G245" s="49"/>
-      <c r="H245" s="51"/>
-      <c r="I245" s="49"/>
-    </row>
-    <row r="246" spans="1:9">
-      <c r="A246" s="52"/>
-      <c r="B246" s="53"/>
-      <c r="C246" s="54"/>
-      <c r="D246" s="53"/>
-      <c r="E246" s="53"/>
+      <c r="H245" s="51" t="s">
+        <v>1106</v>
+      </c>
+      <c r="I245" s="49" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" ht="14">
+      <c r="A246" s="52">
+        <v>46198</v>
+      </c>
+      <c r="B246" s="53" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C246" s="54">
+        <v>1380</v>
+      </c>
+      <c r="D246" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E246" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F246" s="56"/>
       <c r="G246" s="56"/>
-      <c r="H246" s="57"/>
-      <c r="I246" s="53"/>
+      <c r="H246" s="57" t="s">
+        <v>358</v>
+      </c>
+      <c r="I246" s="53" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="247" spans="1:9">
       <c r="A247" s="48"/>
@@ -27579,10 +27679,10 @@
         <v>699</v>
       </c>
       <c r="F120" s="67">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G120" s="67">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H120" s="66">
         <f t="shared" si="9"/>
@@ -27594,14 +27694,14 @@
       </c>
       <c r="J120" s="66">
         <f t="shared" si="10"/>
-        <v>16339.179999999986</v>
+        <v>16758.13333333332</v>
       </c>
       <c r="K120" s="66">
         <f t="shared" si="11"/>
-        <v>2932.6733333333309</v>
+        <v>2513.719999999998</v>
       </c>
       <c r="L120" s="66" t="s">
-        <v>1099</v>
+        <v>1107</v>
       </c>
       <c r="M120" s="66" t="s">
         <v>49</v>
@@ -27611,7 +27711,7 @@
       </c>
       <c r="O120" s="66"/>
       <c r="P120" s="66" t="s">
-        <v>1100</v>
+        <v>1108</v>
       </c>
       <c r="Q120" s="66"/>
       <c r="R120" s="66"/>
@@ -30011,7 +30111,7 @@
         <v>0</v>
       </c>
       <c r="L153" s="69" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="M153" s="69"/>
       <c r="N153" s="69" t="s">
@@ -31175,7 +31275,7 @@
         <v>4189.5</v>
       </c>
       <c r="L175" s="69" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="M175" s="69"/>
       <c r="N175" s="69" t="s">
@@ -31183,7 +31283,7 @@
       </c>
       <c r="O175" s="69"/>
       <c r="P175" s="69" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="Q175" s="69"/>
       <c r="R175" s="69"/>
@@ -31628,10 +31728,10 @@
         <v>1380</v>
       </c>
       <c r="F184" s="81">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G184" s="81">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H184" s="80">
         <f t="shared" ref="H184:H226" si="23">F184+IF(LEN(G184)=0,0,G184)</f>
@@ -31643,14 +31743,14 @@
       </c>
       <c r="J184" s="80">
         <f t="shared" si="21"/>
-        <v>7128</v>
+        <v>9801</v>
       </c>
       <c r="K184" s="80">
         <f t="shared" si="22"/>
-        <v>10692</v>
+        <v>8019</v>
       </c>
       <c r="L184" s="66" t="s">
-        <v>1101</v>
+        <v>1110</v>
       </c>
       <c r="M184" s="66"/>
       <c r="N184" s="66" t="s">
@@ -31702,7 +31802,7 @@
         <v>0</v>
       </c>
       <c r="L185" s="69" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="M185" s="69"/>
       <c r="N185" s="69" t="s">
@@ -31865,7 +31965,7 @@
       <c r="S188" s="66"/>
       <c r="T188" s="66"/>
     </row>
-    <row r="189" spans="1:20" ht="45">
+    <row r="189" spans="1:20" ht="30">
       <c r="A189" s="69" t="s">
         <v>965</v>
       </c>
@@ -31882,10 +31982,10 @@
         <v>1380</v>
       </c>
       <c r="F189" s="79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G189" s="79">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H189" s="78">
         <f t="shared" si="23"/>
@@ -31897,14 +31997,14 @@
       </c>
       <c r="J189" s="78">
         <f t="shared" si="21"/>
-        <v>891</v>
+        <v>1782</v>
       </c>
       <c r="K189" s="78">
         <f t="shared" si="22"/>
-        <v>6237</v>
+        <v>5346</v>
       </c>
       <c r="L189" s="69" t="s">
-        <v>1015</v>
+        <v>1103</v>
       </c>
       <c r="M189" s="69"/>
       <c r="N189" s="69" t="s">
@@ -31912,7 +32012,7 @@
       </c>
       <c r="O189" s="69"/>
       <c r="P189" s="69" t="s">
-        <v>1014</v>
+        <v>1102</v>
       </c>
       <c r="Q189" s="69"/>
       <c r="R189" s="69"/>
@@ -31973,7 +32073,7 @@
         <v>967</v>
       </c>
       <c r="B191" s="66" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="C191" s="66" t="s">
         <v>95</v>
@@ -32012,7 +32112,7 @@
         <v>598</v>
       </c>
       <c r="P191" s="61" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="S191" s="61"/>
       <c r="T191" s="61"/>
@@ -32022,7 +32122,7 @@
         <v>968</v>
       </c>
       <c r="B192" s="69" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="C192" s="69" t="s">
         <v>95</v>
@@ -32061,7 +32161,7 @@
         <v>598</v>
       </c>
       <c r="P192" s="61" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="S192" s="61"/>
       <c r="T192" s="61"/>
@@ -32071,7 +32171,7 @@
         <v>969</v>
       </c>
       <c r="B193" s="66" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="C193" s="66" t="s">
         <v>95</v>
@@ -32110,7 +32210,7 @@
         <v>598</v>
       </c>
       <c r="P193" s="61" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="S193" s="61"/>
       <c r="T193" s="61"/>
@@ -32120,7 +32220,7 @@
         <v>970</v>
       </c>
       <c r="B194" s="66" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="C194" s="66" t="s">
         <v>95</v>
@@ -32159,7 +32259,7 @@
         <v>598</v>
       </c>
       <c r="P194" s="61" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="S194" s="61"/>
       <c r="T194" s="61"/>
@@ -32169,7 +32269,7 @@
         <v>971</v>
       </c>
       <c r="B195" s="69" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="C195" s="69" t="s">
         <v>95</v>
@@ -32203,14 +32303,14 @@
         <v>5467</v>
       </c>
       <c r="L195" s="69" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="M195" s="69"/>
       <c r="N195" s="61" t="s">
         <v>510</v>
       </c>
       <c r="P195" s="61" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="S195" s="61"/>
       <c r="T195" s="61"/>
@@ -32220,7 +32320,7 @@
         <v>972</v>
       </c>
       <c r="B196" s="66" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="C196" s="66" t="s">
         <v>95</v>
@@ -32259,7 +32359,7 @@
         <v>598</v>
       </c>
       <c r="P196" s="61" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="S196" s="61"/>
       <c r="T196" s="61"/>
@@ -32269,7 +32369,7 @@
         <v>973</v>
       </c>
       <c r="B197" s="69" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="C197" s="69" t="s">
         <v>95</v>
@@ -32308,7 +32408,7 @@
         <v>598</v>
       </c>
       <c r="P197" s="61" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="S197" s="61"/>
       <c r="T197" s="61"/>
@@ -32318,7 +32418,7 @@
         <v>974</v>
       </c>
       <c r="B198" s="66" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="C198" s="66" t="s">
         <v>95</v>
@@ -32357,7 +32457,7 @@
         <v>598</v>
       </c>
       <c r="P198" s="61" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="S198" s="61"/>
       <c r="T198" s="61"/>
@@ -32367,7 +32467,7 @@
         <v>975</v>
       </c>
       <c r="B199" s="66" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="C199" s="66" t="s">
         <v>95</v>
@@ -32406,7 +32506,7 @@
         <v>598</v>
       </c>
       <c r="P199" s="61" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="S199" s="61"/>
       <c r="T199" s="61"/>
@@ -32416,7 +32516,7 @@
         <v>976</v>
       </c>
       <c r="B200" s="69" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="C200" s="69" t="s">
         <v>95</v>
@@ -32450,14 +32550,14 @@
         <v>1732</v>
       </c>
       <c r="L200" s="66" t="s">
-        <v>1104</v>
+        <v>1097</v>
       </c>
       <c r="M200" s="66"/>
       <c r="N200" s="61" t="s">
         <v>510</v>
       </c>
       <c r="P200" s="61" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="S200" s="61"/>
       <c r="T200" s="61"/>
@@ -32467,7 +32567,7 @@
         <v>977</v>
       </c>
       <c r="B201" s="66" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="C201" s="66" t="s">
         <v>95</v>
@@ -32501,14 +32601,14 @@
         <v>724</v>
       </c>
       <c r="L201" s="69" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="M201" s="69"/>
       <c r="N201" s="61" t="s">
         <v>510</v>
       </c>
       <c r="P201" s="61" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="S201" s="61"/>
       <c r="T201" s="61"/>
@@ -32518,7 +32618,7 @@
         <v>978</v>
       </c>
       <c r="B202" s="69" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="C202" s="69" t="s">
         <v>95</v>
@@ -32557,7 +32657,7 @@
         <v>598</v>
       </c>
       <c r="P202" s="61" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="S202" s="61"/>
       <c r="T202" s="61"/>
@@ -32567,7 +32667,7 @@
         <v>979</v>
       </c>
       <c r="B203" s="66" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="C203" s="66" t="s">
         <v>95</v>
@@ -32601,14 +32701,14 @@
         <v>0</v>
       </c>
       <c r="L203" s="69" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="M203" s="69"/>
       <c r="N203" s="61" t="s">
         <v>425</v>
       </c>
       <c r="P203" s="61" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="S203" s="61"/>
       <c r="T203" s="61"/>
@@ -32618,7 +32718,7 @@
         <v>980</v>
       </c>
       <c r="B204" s="66" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="C204" s="66" t="s">
         <v>95</v>
@@ -32652,14 +32752,14 @@
         <v>1760</v>
       </c>
       <c r="L204" s="66" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="M204" s="66"/>
       <c r="N204" s="61" t="s">
         <v>510</v>
       </c>
       <c r="P204" s="61" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="S204" s="61"/>
       <c r="T204" s="61"/>
@@ -32669,7 +32769,7 @@
         <v>981</v>
       </c>
       <c r="B205" s="69" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="C205" s="69" t="s">
         <v>95</v>
@@ -32703,14 +32803,14 @@
         <v>1522</v>
       </c>
       <c r="L205" s="69" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="M205" s="69"/>
       <c r="N205" s="61" t="s">
         <v>598</v>
       </c>
       <c r="P205" s="61" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="S205" s="61"/>
       <c r="T205" s="61"/>
@@ -32720,7 +32820,7 @@
         <v>982</v>
       </c>
       <c r="B206" s="66" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="C206" s="66" t="s">
         <v>95</v>
@@ -32759,7 +32859,7 @@
         <v>598</v>
       </c>
       <c r="P206" s="61" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="S206" s="61"/>
       <c r="T206" s="61"/>
@@ -32769,7 +32869,7 @@
         <v>983</v>
       </c>
       <c r="B207" s="69" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="C207" s="69" t="s">
         <v>95</v>
@@ -32803,14 +32903,14 @@
         <v>3312</v>
       </c>
       <c r="L207" s="69" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="M207" s="69"/>
       <c r="N207" s="61" t="s">
         <v>510</v>
       </c>
       <c r="P207" s="61" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="S207" s="61"/>
       <c r="T207" s="61"/>
@@ -32820,7 +32920,7 @@
         <v>984</v>
       </c>
       <c r="B208" s="66" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="C208" s="66" t="s">
         <v>95</v>
@@ -32859,7 +32959,7 @@
         <v>598</v>
       </c>
       <c r="P208" s="61" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="S208" s="61"/>
       <c r="T208" s="61"/>
@@ -32869,7 +32969,7 @@
         <v>985</v>
       </c>
       <c r="B209" s="66" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C209" s="66" t="s">
         <v>95</v>
@@ -32908,7 +33008,7 @@
         <v>598</v>
       </c>
       <c r="P209" s="61" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="S209" s="61"/>
       <c r="T209" s="61"/>
@@ -32918,7 +33018,7 @@
         <v>986</v>
       </c>
       <c r="B210" s="69" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="C210" s="69" t="s">
         <v>95</v>
@@ -32957,7 +33057,7 @@
         <v>598</v>
       </c>
       <c r="P210" s="61" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="S210" s="61"/>
       <c r="T210" s="61"/>
@@ -32967,7 +33067,7 @@
         <v>987</v>
       </c>
       <c r="B211" s="66" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="C211" s="66" t="s">
         <v>95</v>
@@ -33006,7 +33106,7 @@
         <v>598</v>
       </c>
       <c r="P211" s="61" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="S211" s="61"/>
       <c r="T211" s="61"/>
@@ -37487,15 +37587,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>212623</v>
+        <v>212783</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>61436.333333333343</v>
+        <v>61543</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -37503,7 +37603,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>61436.333333333343</v>
+        <v>61543</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -37511,7 +37611,7 @@
       </c>
       <c r="H8" s="88">
         <f>F8-G8</f>
-        <v>43132.993333333347</v>
+        <v>43239.66</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -37524,11 +37624,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>57150.333333333343</v>
+        <v>57097</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -37536,7 +37636,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>57150.333333333343</v>
+        <v>57097</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -37544,7 +37644,7 @@
       </c>
       <c r="H9" s="89">
         <f>F9-G9</f>
-        <v>15511.003333333341</v>
+        <v>15457.669999999998</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -37557,11 +37657,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>151186.66666666666</v>
+        <v>151240</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-118586.66666666666</v>
+        <v>-118640</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -37569,7 +37669,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-118586.66666666666</v>
+        <v>-118640</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -37577,7 +37677,7 @@
       </c>
       <c r="H10" s="88">
         <f>F10-G10</f>
-        <v>-58643.996666666659</v>
+        <v>-58697.33</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="90" customFormat="1" ht="15.75" customHeight="1">
@@ -37994,7 +38094,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>331518</v>
+        <v>341737</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -38002,11 +38102,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>132917.24479999999</v>
+        <v>136324.25939999998</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>198600.75520000001</v>
+        <v>205412.74060000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38014,7 +38114,7 @@
       </c>
       <c r="G4" s="88">
         <f>E4+F4</f>
-        <v>61290.729200000002</v>
+        <v>68102.714600000007</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -38031,11 +38131,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>132837.5104</v>
+        <v>136242.48120000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-78213.510399999999</v>
+        <v>-81618.481200000009</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38043,7 +38143,7 @@
       </c>
       <c r="G5" s="89">
         <f>E5+F5</f>
-        <v>-6626.4683999999979</v>
+        <v>-10031.439200000008</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -38060,11 +38160,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>132917.24479999999</v>
+        <v>136324.25939999998</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-120387.24479999999</v>
+        <v>-123794.25939999998</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38072,7 +38172,7 @@
       </c>
       <c r="G6" s="88">
         <f>E6+F6</f>
-        <v>-54664.260799999975</v>
+        <v>-58071.27539999997</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>